<commit_message>
Last minute coherence corrections among different correlated files.
</commit_message>
<xml_diff>
--- a/status/Gantt_live_11DP-C.xlsx
+++ b/status/Gantt_live_11DP-C.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ettore/AI/ClaudeCode/BBI/IB/IB_Project/Submission/Freshman_version/plan_v2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF5DA5B1-C292-8642-BDA1-8425A97C2829}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35C98A9B-1FAA-9C4F-9FD4-4B963B1F29F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="30240" windowHeight="19640" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="17980" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Read me" sheetId="1" r:id="rId1"/>
@@ -252,7 +252,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="693" uniqueCount="404">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="698" uniqueCount="409">
   <si>
     <t>Project Status · Group 11DP-C · Pyruvate Kinase Deficiency</t>
   </si>
@@ -350,30 +350,48 @@
     <t>1.1 Review and commit the introduction (PKD_1); create the folders report/, status/, gantt/, and references/</t>
   </si>
   <si>
+    <t>Introduction committed by Ettore on 9 Oct; the folders gantt/, status/, references/, and report/ were created by Leo and Bruno on 8 Oct.</t>
+  </si>
+  <si>
+    <t>1.2 Review and commit the overview and team section (PKD_2); submit the repository URL on Moodle</t>
+  </si>
+  <si>
+    <t>In progress</t>
+  </si>
+  <si>
+    <t>PKD_2 committed by Aarón on 8 Oct (roles of Bruno and Leo swapped by team decision); Moodle URL submission to be confirmed.</t>
+  </si>
+  <si>
+    <t>1.3 Review and commit the Gantt chart (PKD_3)</t>
+  </si>
+  <si>
+    <t>Bruno</t>
+  </si>
+  <si>
+    <t>Committed by Leo on 8 Oct and edited by Pol; owner after the role swap: Bruno.</t>
+  </si>
+  <si>
+    <t>1.4 Review and commit the task details (PKD_4)</t>
+  </si>
+  <si>
+    <t>Pol</t>
+  </si>
+  <si>
+    <t>Committed by Pol on 8 Oct; owner columns corrected for the role swap.</t>
+  </si>
+  <si>
+    <t>1.5 Review and commit the risk analysis and references (PKD_5, PKD_6)</t>
+  </si>
+  <si>
+    <t>Committed by Bruno (PKD_6 on 8 Oct, PKD_5 on 9 Oct), references updated by Ettore on 9 Oct; owner after the role swap: Leo.</t>
+  </si>
+  <si>
+    <t>1.6 Create the Project Status document</t>
+  </si>
+  <si>
     <t>Pending</t>
   </si>
   <si>
-    <t>1.2 Review and commit the overview and team section (PKD_2); submit the repository URL on Moodle</t>
-  </si>
-  <si>
-    <t>1.3 Review and commit the Gantt chart (PKD_3)</t>
-  </si>
-  <si>
-    <t>1.4 Review and commit the task details (PKD_4)</t>
-  </si>
-  <si>
-    <t>Pol</t>
-  </si>
-  <si>
-    <t>1.5 Review and commit the risk analysis and references (PKD_5, PKD_6)</t>
-  </si>
-  <si>
-    <t>Bruno</t>
-  </si>
-  <si>
-    <t>1.6 Create the Project Status document</t>
-  </si>
-  <si>
     <t>1.7 Weekly status update and team meeting (Fridays 16 and 23 Oct)</t>
   </si>
   <si>
@@ -507,9 +525,6 @@
   </si>
   <si>
     <t>A problem occurred; describe it and the workaround in Notes</t>
-  </si>
-  <si>
-    <t>In progress</t>
   </si>
   <si>
     <t>Started; Real Start Date filled</t>
@@ -1231,19 +1246,19 @@
     <t>Bruno Carrasquilla</t>
   </si>
   <si>
+    <t>Sequence Analyst</t>
+  </si>
+  <si>
+    <t>Ettore Colombo</t>
+  </si>
+  <si>
+    <t>Project Manager</t>
+  </si>
+  <si>
+    <t>Leo Nader Al Hourani</t>
+  </si>
+  <si>
     <t>Data and GitHub Manager</t>
-  </si>
-  <si>
-    <t>Ettore Colombo</t>
-  </si>
-  <si>
-    <t>Project Manager</t>
-  </si>
-  <si>
-    <t>Leo Nader Al Hourani</t>
-  </si>
-  <si>
-    <t>Sequence Analyst</t>
   </si>
   <si>
     <t>Pol Monllau</t>
@@ -1592,14 +1607,14 @@
     <font>
       <b/>
       <sz val="10"/>
-      <color rgb="FF00A6FB"/>
+      <color rgb="FF8AC926"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
-      <color rgb="FF8AC926"/>
+      <color rgb="FF00A6FB"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -1997,10 +2012,10 @@
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -2996,12 +3011,12 @@
   <sheetData>
     <row r="1" spans="1:1" ht="19" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
@@ -3009,37 +3024,37 @@
     </row>
     <row r="4" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
     </row>
     <row r="6" spans="1:1" ht="28" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
     </row>
     <row r="8" spans="1:1" ht="28" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
     </row>
     <row r="10" spans="1:1" ht="28" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.2">
@@ -3047,22 +3062,22 @@
     </row>
     <row r="12" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A13" s="5" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A14" s="5" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
     </row>
     <row r="15" spans="1:1" ht="28" x14ac:dyDescent="0.2">
       <c r="A15" s="5" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.2">
@@ -3070,17 +3085,17 @@
     </row>
     <row r="17" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
     </row>
     <row r="18" spans="1:1" ht="28" x14ac:dyDescent="0.2">
       <c r="A18" s="5" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A19" s="5" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.2">
@@ -3088,22 +3103,22 @@
     </row>
     <row r="21" spans="1:1" ht="17" x14ac:dyDescent="0.2">
       <c r="A21" s="4" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="22" spans="1:1" ht="28" x14ac:dyDescent="0.2">
       <c r="A22" s="5" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
     </row>
     <row r="23" spans="1:1" ht="56" x14ac:dyDescent="0.2">
       <c r="A23" s="5" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A26" s="6" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
     </row>
   </sheetData>
@@ -3136,7 +3151,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="9">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="C2" s="10" t="s">
         <v>2</v>
@@ -3459,12 +3474,18 @@
         <f>Tasks!I16</f>
         <v>46304</v>
       </c>
-      <c r="E16" s="17"/>
-      <c r="F16" s="17"/>
+      <c r="E16" s="17">
+        <v>46304</v>
+      </c>
+      <c r="F16" s="17">
+        <v>46304</v>
+      </c>
       <c r="G16" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="H16" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="H16" s="19"/>
     </row>
     <row r="17" spans="1:8" ht="28" x14ac:dyDescent="0.2">
       <c r="A17" s="14" t="s">
@@ -3481,19 +3502,23 @@
         <f>Tasks!I17</f>
         <v>46304</v>
       </c>
-      <c r="E17" s="17"/>
+      <c r="E17" s="17">
+        <v>46303</v>
+      </c>
       <c r="F17" s="17"/>
       <c r="G17" s="18" t="s">
-        <v>32</v>
-      </c>
-      <c r="H17" s="19"/>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+        <v>34</v>
+      </c>
+      <c r="H17" s="19" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="28" x14ac:dyDescent="0.2">
       <c r="A18" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="B18" s="15" t="s">
-        <v>13</v>
+        <v>36</v>
+      </c>
+      <c r="B18" s="25" t="s">
+        <v>37</v>
       </c>
       <c r="C18" s="16">
         <f>Tasks!H18</f>
@@ -3503,19 +3528,25 @@
         <f>Tasks!I18</f>
         <v>46304</v>
       </c>
-      <c r="E18" s="17"/>
-      <c r="F18" s="17"/>
+      <c r="E18" s="17">
+        <v>46303</v>
+      </c>
+      <c r="F18" s="17">
+        <v>46303</v>
+      </c>
       <c r="G18" s="18" t="s">
-        <v>32</v>
-      </c>
-      <c r="H18" s="19"/>
+        <v>14</v>
+      </c>
+      <c r="H18" s="19" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="B19" s="25" t="s">
-        <v>36</v>
+        <v>39</v>
+      </c>
+      <c r="B19" s="26" t="s">
+        <v>40</v>
       </c>
       <c r="C19" s="16">
         <f>Tasks!H19</f>
@@ -3525,19 +3556,25 @@
         <f>Tasks!I19</f>
         <v>46304</v>
       </c>
-      <c r="E19" s="17"/>
-      <c r="F19" s="17"/>
+      <c r="E19" s="17">
+        <v>46303</v>
+      </c>
+      <c r="F19" s="17">
+        <v>46303</v>
+      </c>
       <c r="G19" s="18" t="s">
-        <v>32</v>
-      </c>
-      <c r="H19" s="19"/>
+        <v>14</v>
+      </c>
+      <c r="H19" s="19" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="20" spans="1:8" ht="28" x14ac:dyDescent="0.2">
       <c r="A20" s="14" t="s">
-        <v>37</v>
-      </c>
-      <c r="B20" s="26" t="s">
-        <v>38</v>
+        <v>42</v>
+      </c>
+      <c r="B20" s="15" t="s">
+        <v>13</v>
       </c>
       <c r="C20" s="16">
         <f>Tasks!H20</f>
@@ -3547,16 +3584,22 @@
         <f>Tasks!I20</f>
         <v>46304</v>
       </c>
-      <c r="E20" s="17"/>
-      <c r="F20" s="17"/>
+      <c r="E20" s="17">
+        <v>46303</v>
+      </c>
+      <c r="F20" s="17">
+        <v>46304</v>
+      </c>
       <c r="G20" s="18" t="s">
-        <v>32</v>
-      </c>
-      <c r="H20" s="19"/>
+        <v>14</v>
+      </c>
+      <c r="H20" s="19" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21" s="14" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="B21" s="20" t="s">
         <v>17</v>
@@ -3572,13 +3615,13 @@
       <c r="E21" s="17"/>
       <c r="F21" s="17"/>
       <c r="G21" s="18" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="H21" s="19"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" s="14" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="B22" s="20" t="s">
         <v>17</v>
@@ -3594,13 +3637,13 @@
       <c r="E22" s="17"/>
       <c r="F22" s="17"/>
       <c r="G22" s="18" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="H22" s="19"/>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A23" s="14" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="B23" s="20" t="s">
         <v>17</v>
@@ -3616,13 +3659,13 @@
       <c r="E23" s="17"/>
       <c r="F23" s="17"/>
       <c r="G23" s="18" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="H23" s="19"/>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A24" s="14" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="B24" s="20" t="s">
         <v>17</v>
@@ -3638,13 +3681,13 @@
       <c r="E24" s="17"/>
       <c r="F24" s="17"/>
       <c r="G24" s="18" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="H24" s="19"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A25" s="27" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="B25" s="28"/>
       <c r="C25" s="28"/>
@@ -3656,10 +3699,10 @@
     </row>
     <row r="26" spans="1:8" ht="42" x14ac:dyDescent="0.2">
       <c r="A26" s="14" t="s">
-        <v>44</v>
-      </c>
-      <c r="B26" s="15" t="s">
-        <v>13</v>
+        <v>50</v>
+      </c>
+      <c r="B26" s="25" t="s">
+        <v>37</v>
       </c>
       <c r="C26" s="16">
         <f>Tasks!H26</f>
@@ -3672,16 +3715,16 @@
       <c r="E26" s="17"/>
       <c r="F26" s="17"/>
       <c r="G26" s="18" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="H26" s="19"/>
     </row>
     <row r="27" spans="1:8" ht="28" x14ac:dyDescent="0.2">
       <c r="A27" s="14" t="s">
-        <v>45</v>
-      </c>
-      <c r="B27" s="26" t="s">
-        <v>38</v>
+        <v>51</v>
+      </c>
+      <c r="B27" s="15" t="s">
+        <v>13</v>
       </c>
       <c r="C27" s="16">
         <f>Tasks!H27</f>
@@ -3694,16 +3737,16 @@
       <c r="E27" s="17"/>
       <c r="F27" s="17"/>
       <c r="G27" s="18" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="H27" s="19"/>
     </row>
     <row r="28" spans="1:8" ht="28" x14ac:dyDescent="0.2">
       <c r="A28" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="B28" s="26" t="s">
-        <v>38</v>
+        <v>52</v>
+      </c>
+      <c r="B28" s="15" t="s">
+        <v>13</v>
       </c>
       <c r="C28" s="16">
         <f>Tasks!H28</f>
@@ -3716,13 +3759,13 @@
       <c r="E28" s="17"/>
       <c r="F28" s="17"/>
       <c r="G28" s="18" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="H28" s="19"/>
     </row>
     <row r="29" spans="1:8" ht="28" x14ac:dyDescent="0.2">
       <c r="A29" s="14" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="B29" s="22" t="s">
         <v>23</v>
@@ -3738,16 +3781,16 @@
       <c r="E29" s="17"/>
       <c r="F29" s="17"/>
       <c r="G29" s="18" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="H29" s="19"/>
     </row>
     <row r="30" spans="1:8" ht="28" x14ac:dyDescent="0.2">
       <c r="A30" s="14" t="s">
-        <v>48</v>
-      </c>
-      <c r="B30" s="26" t="s">
-        <v>38</v>
+        <v>54</v>
+      </c>
+      <c r="B30" s="15" t="s">
+        <v>13</v>
       </c>
       <c r="C30" s="16">
         <f>Tasks!H30</f>
@@ -3760,16 +3803,16 @@
       <c r="E30" s="17"/>
       <c r="F30" s="17"/>
       <c r="G30" s="18" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="H30" s="19"/>
     </row>
     <row r="31" spans="1:8" ht="28" x14ac:dyDescent="0.2">
       <c r="A31" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="B31" s="25" t="s">
-        <v>36</v>
+        <v>55</v>
+      </c>
+      <c r="B31" s="26" t="s">
+        <v>40</v>
       </c>
       <c r="C31" s="16">
         <f>Tasks!H31</f>
@@ -3782,16 +3825,16 @@
       <c r="E31" s="17"/>
       <c r="F31" s="17"/>
       <c r="G31" s="18" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="H31" s="19"/>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A32" s="14" t="s">
-        <v>50</v>
-      </c>
-      <c r="B32" s="26" t="s">
-        <v>38</v>
+        <v>56</v>
+      </c>
+      <c r="B32" s="15" t="s">
+        <v>13</v>
       </c>
       <c r="C32" s="16">
         <f>Tasks!H32</f>
@@ -3804,13 +3847,13 @@
       <c r="E32" s="17"/>
       <c r="F32" s="17"/>
       <c r="G32" s="18" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="H32" s="19"/>
     </row>
     <row r="33" spans="1:8" ht="28" x14ac:dyDescent="0.2">
       <c r="A33" s="14" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="B33" s="20" t="s">
         <v>17</v>
@@ -3826,13 +3869,13 @@
       <c r="E33" s="17"/>
       <c r="F33" s="17"/>
       <c r="G33" s="18" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="H33" s="19"/>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A34" s="29" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="B34" s="30"/>
       <c r="C34" s="30"/>
@@ -3844,10 +3887,10 @@
     </row>
     <row r="35" spans="1:8" ht="28" x14ac:dyDescent="0.2">
       <c r="A35" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="B35" s="15" t="s">
-        <v>13</v>
+        <v>59</v>
+      </c>
+      <c r="B35" s="25" t="s">
+        <v>37</v>
       </c>
       <c r="C35" s="16">
         <f>Tasks!H35</f>
@@ -3860,16 +3903,16 @@
       <c r="E35" s="17"/>
       <c r="F35" s="17"/>
       <c r="G35" s="18" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="H35" s="19"/>
     </row>
     <row r="36" spans="1:8" ht="28" x14ac:dyDescent="0.2">
       <c r="A36" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="B36" s="15" t="s">
-        <v>13</v>
+        <v>60</v>
+      </c>
+      <c r="B36" s="25" t="s">
+        <v>37</v>
       </c>
       <c r="C36" s="16">
         <f>Tasks!H36</f>
@@ -3882,16 +3925,16 @@
       <c r="E36" s="17"/>
       <c r="F36" s="17"/>
       <c r="G36" s="18" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="H36" s="19"/>
     </row>
     <row r="37" spans="1:8" ht="28" x14ac:dyDescent="0.2">
       <c r="A37" s="14" t="s">
-        <v>55</v>
-      </c>
-      <c r="B37" s="25" t="s">
-        <v>36</v>
+        <v>61</v>
+      </c>
+      <c r="B37" s="26" t="s">
+        <v>40</v>
       </c>
       <c r="C37" s="16">
         <f>Tasks!H37</f>
@@ -3904,16 +3947,16 @@
       <c r="E37" s="17"/>
       <c r="F37" s="17"/>
       <c r="G37" s="18" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="H37" s="19"/>
     </row>
     <row r="38" spans="1:8" ht="28" x14ac:dyDescent="0.2">
       <c r="A38" s="14" t="s">
-        <v>56</v>
-      </c>
-      <c r="B38" s="25" t="s">
-        <v>36</v>
+        <v>62</v>
+      </c>
+      <c r="B38" s="26" t="s">
+        <v>40</v>
       </c>
       <c r="C38" s="16">
         <f>Tasks!H38</f>
@@ -3926,16 +3969,16 @@
       <c r="E38" s="17"/>
       <c r="F38" s="17"/>
       <c r="G38" s="18" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="H38" s="19"/>
     </row>
     <row r="39" spans="1:8" ht="28" x14ac:dyDescent="0.2">
       <c r="A39" s="14" t="s">
-        <v>57</v>
-      </c>
-      <c r="B39" s="25" t="s">
-        <v>36</v>
+        <v>63</v>
+      </c>
+      <c r="B39" s="26" t="s">
+        <v>40</v>
       </c>
       <c r="C39" s="16">
         <f>Tasks!H39</f>
@@ -3948,13 +3991,13 @@
       <c r="E39" s="17"/>
       <c r="F39" s="17"/>
       <c r="G39" s="18" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="H39" s="19"/>
     </row>
     <row r="40" spans="1:8" ht="28" x14ac:dyDescent="0.2">
       <c r="A40" s="14" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="B40" s="22" t="s">
         <v>23</v>
@@ -3970,13 +4013,13 @@
       <c r="E40" s="17"/>
       <c r="F40" s="17"/>
       <c r="G40" s="18" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="H40" s="19"/>
     </row>
     <row r="41" spans="1:8" ht="28" x14ac:dyDescent="0.2">
       <c r="A41" s="14" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="B41" s="22" t="s">
         <v>23</v>
@@ -3992,13 +4035,13 @@
       <c r="E41" s="17"/>
       <c r="F41" s="17"/>
       <c r="G41" s="18" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="H41" s="19"/>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A42" s="14" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="B42" s="20" t="s">
         <v>17</v>
@@ -4014,16 +4057,16 @@
       <c r="E42" s="17"/>
       <c r="F42" s="17"/>
       <c r="G42" s="18" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="H42" s="19"/>
     </row>
     <row r="43" spans="1:8" ht="42" x14ac:dyDescent="0.2">
       <c r="A43" s="14" t="s">
-        <v>61</v>
-      </c>
-      <c r="B43" s="26" t="s">
-        <v>38</v>
+        <v>67</v>
+      </c>
+      <c r="B43" s="15" t="s">
+        <v>13</v>
       </c>
       <c r="C43" s="16">
         <f>Tasks!H43</f>
@@ -4036,13 +4079,13 @@
       <c r="E43" s="17"/>
       <c r="F43" s="17"/>
       <c r="G43" s="18" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="H43" s="19"/>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A44" s="31" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="B44" s="32"/>
       <c r="C44" s="32"/>
@@ -4054,7 +4097,7 @@
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A45" s="14" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="B45" s="22" t="s">
         <v>23</v>
@@ -4070,16 +4113,16 @@
       <c r="E45" s="17"/>
       <c r="F45" s="17"/>
       <c r="G45" s="18" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="H45" s="19"/>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A46" s="14" t="s">
-        <v>64</v>
-      </c>
-      <c r="B46" s="26" t="s">
-        <v>38</v>
+        <v>70</v>
+      </c>
+      <c r="B46" s="15" t="s">
+        <v>13</v>
       </c>
       <c r="C46" s="16">
         <f>Tasks!H46</f>
@@ -4092,16 +4135,16 @@
       <c r="E46" s="17"/>
       <c r="F46" s="17"/>
       <c r="G46" s="18" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="H46" s="19"/>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A47" s="14" t="s">
-        <v>65</v>
-      </c>
-      <c r="B47" s="15" t="s">
-        <v>13</v>
+        <v>71</v>
+      </c>
+      <c r="B47" s="25" t="s">
+        <v>37</v>
       </c>
       <c r="C47" s="16">
         <f>Tasks!H47</f>
@@ -4114,16 +4157,16 @@
       <c r="E47" s="17"/>
       <c r="F47" s="17"/>
       <c r="G47" s="18" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="H47" s="19"/>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A48" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="B48" s="25" t="s">
-        <v>36</v>
+        <v>72</v>
+      </c>
+      <c r="B48" s="26" t="s">
+        <v>40</v>
       </c>
       <c r="C48" s="16">
         <f>Tasks!H48</f>
@@ -4136,13 +4179,13 @@
       <c r="E48" s="17"/>
       <c r="F48" s="17"/>
       <c r="G48" s="18" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="H48" s="19"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A49" s="14" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="B49" s="20" t="s">
         <v>17</v>
@@ -4158,13 +4201,13 @@
       <c r="E49" s="17"/>
       <c r="F49" s="17"/>
       <c r="G49" s="18" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="H49" s="19"/>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A50" s="14" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="B50" s="22" t="s">
         <v>23</v>
@@ -4180,16 +4223,16 @@
       <c r="E50" s="17"/>
       <c r="F50" s="17"/>
       <c r="G50" s="18" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="H50" s="19"/>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A51" s="14" t="s">
-        <v>69</v>
-      </c>
-      <c r="B51" s="15" t="s">
-        <v>13</v>
+        <v>75</v>
+      </c>
+      <c r="B51" s="25" t="s">
+        <v>37</v>
       </c>
       <c r="C51" s="16">
         <f>Tasks!H51</f>
@@ -4202,16 +4245,16 @@
       <c r="E51" s="17"/>
       <c r="F51" s="17"/>
       <c r="G51" s="18" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="H51" s="19"/>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A52" s="14" t="s">
-        <v>70</v>
-      </c>
-      <c r="B52" s="26" t="s">
-        <v>38</v>
+        <v>76</v>
+      </c>
+      <c r="B52" s="15" t="s">
+        <v>13</v>
       </c>
       <c r="C52" s="16">
         <f>Tasks!H52</f>
@@ -4224,13 +4267,13 @@
       <c r="E52" s="17"/>
       <c r="F52" s="17"/>
       <c r="G52" s="18" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="H52" s="19"/>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A53" s="14" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="B53" s="22" t="s">
         <v>23</v>
@@ -4246,13 +4289,13 @@
       <c r="E53" s="17"/>
       <c r="F53" s="17"/>
       <c r="G53" s="18" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="H53" s="19"/>
     </row>
     <row r="54" spans="1:8" ht="28" x14ac:dyDescent="0.2">
       <c r="A54" s="14" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="B54" s="22" t="s">
         <v>23</v>
@@ -4268,16 +4311,16 @@
       <c r="E54" s="17"/>
       <c r="F54" s="17"/>
       <c r="G54" s="18" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="H54" s="19"/>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A55" s="14" t="s">
-        <v>73</v>
-      </c>
-      <c r="B55" s="26" t="s">
-        <v>38</v>
+        <v>79</v>
+      </c>
+      <c r="B55" s="15" t="s">
+        <v>13</v>
       </c>
       <c r="C55" s="16">
         <f>Tasks!H55</f>
@@ -4290,13 +4333,13 @@
       <c r="E55" s="17"/>
       <c r="F55" s="17"/>
       <c r="G55" s="18" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="H55" s="19"/>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A56" s="14" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="B56" s="20" t="s">
         <v>17</v>
@@ -4312,16 +4355,16 @@
       <c r="E56" s="17"/>
       <c r="F56" s="17"/>
       <c r="G56" s="18" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="H56" s="19"/>
     </row>
     <row r="57" spans="1:8" ht="28" x14ac:dyDescent="0.2">
       <c r="A57" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="B57" s="15" t="s">
-        <v>13</v>
+        <v>81</v>
+      </c>
+      <c r="B57" s="25" t="s">
+        <v>37</v>
       </c>
       <c r="C57" s="16">
         <f>Tasks!H57</f>
@@ -4334,16 +4377,16 @@
       <c r="E57" s="17"/>
       <c r="F57" s="17"/>
       <c r="G57" s="18" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="H57" s="19"/>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A58" s="14" t="s">
-        <v>76</v>
-      </c>
-      <c r="B58" s="25" t="s">
-        <v>36</v>
+        <v>82</v>
+      </c>
+      <c r="B58" s="26" t="s">
+        <v>40</v>
       </c>
       <c r="C58" s="16">
         <f>Tasks!H58</f>
@@ -4356,16 +4399,16 @@
       <c r="E58" s="17"/>
       <c r="F58" s="17"/>
       <c r="G58" s="18" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="H58" s="19"/>
     </row>
     <row r="59" spans="1:8" ht="28" x14ac:dyDescent="0.2">
       <c r="A59" s="14" t="s">
-        <v>77</v>
-      </c>
-      <c r="B59" s="26" t="s">
-        <v>38</v>
+        <v>83</v>
+      </c>
+      <c r="B59" s="15" t="s">
+        <v>13</v>
       </c>
       <c r="C59" s="16">
         <f>Tasks!H59</f>
@@ -4378,16 +4421,16 @@
       <c r="E59" s="17"/>
       <c r="F59" s="17"/>
       <c r="G59" s="18" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="H59" s="19"/>
     </row>
     <row r="60" spans="1:8" ht="28" x14ac:dyDescent="0.2">
       <c r="A60" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="B60" s="15" t="s">
-        <v>13</v>
+        <v>84</v>
+      </c>
+      <c r="B60" s="25" t="s">
+        <v>37</v>
       </c>
       <c r="C60" s="16">
         <f>Tasks!H60</f>
@@ -4400,21 +4443,21 @@
       <c r="E60" s="17"/>
       <c r="F60" s="17"/>
       <c r="G60" s="18" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="H60" s="19"/>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A62" s="33" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A63" s="34" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="B63" s="35" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.2">
@@ -4422,44 +4465,44 @@
         <v>14</v>
       </c>
       <c r="B64" s="35" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A65" s="37" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="B65" s="35" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A66" s="38" t="s">
-        <v>85</v>
+        <v>34</v>
       </c>
       <c r="B66" s="35" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A67" s="39" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="B67" s="35" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A68" s="40" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="B68" s="35" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A70" s="10" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
     </row>
   </sheetData>
@@ -4530,12 +4573,12 @@
   <sheetData>
     <row r="1" spans="1:50" ht="17" x14ac:dyDescent="0.2">
       <c r="A1" s="41" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A2" s="10" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
     </row>
     <row r="3" spans="1:50" x14ac:dyDescent="0.2">
@@ -4594,43 +4637,43 @@
     </row>
     <row r="4" spans="1:50" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="11" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="C4" s="11" t="s">
         <v>3</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="F4" s="11" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="G4" s="11" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="H4" s="11" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="I4" s="11" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="J4" s="11" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="K4" s="11" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="L4" s="11" t="s">
         <v>9</v>
       </c>
       <c r="M4" s="11" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="N4" s="42">
         <v>46282</v>
@@ -4741,15 +4784,15 @@
         <v>46331</v>
       </c>
       <c r="AX4" s="11" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
     </row>
     <row r="5" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A5" s="12" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="C5" s="13" t="s">
         <v>11</v>
@@ -4812,13 +4855,13 @@
     </row>
     <row r="6" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A6" s="45" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="B6" s="45" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="C6" s="45" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="D6" s="46" t="s">
         <v>13</v>
@@ -4998,18 +5041,18 @@
         <v/>
       </c>
       <c r="AX6" s="49" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
     </row>
     <row r="7" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A7" s="45" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="B7" s="45" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="C7" s="45" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="D7" s="50" t="s">
         <v>17</v>
@@ -5189,18 +5232,18 @@
         <v/>
       </c>
       <c r="AX7" s="49" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
     </row>
     <row r="8" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A8" s="45" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="B8" s="45" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="C8" s="45" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="D8" s="51" t="s">
         <v>19</v>
@@ -5380,18 +5423,18 @@
         <v/>
       </c>
       <c r="AX8" s="49" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
     </row>
     <row r="9" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A9" s="45" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="B9" s="45" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="C9" s="45" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="D9" s="51" t="s">
         <v>19</v>
@@ -5571,18 +5614,18 @@
         <v/>
       </c>
       <c r="AX9" s="49" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
     </row>
     <row r="10" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A10" s="45" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="B10" s="45" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="C10" s="45" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="D10" s="52" t="s">
         <v>23</v>
@@ -5762,18 +5805,18 @@
         <v/>
       </c>
       <c r="AX10" s="49" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
     </row>
     <row r="11" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A11" s="45" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="B11" s="45" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="C11" s="45" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="D11" s="51" t="s">
         <v>19</v>
@@ -5953,18 +5996,18 @@
         <v/>
       </c>
       <c r="AX11" s="49" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
     </row>
     <row r="12" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A12" s="45" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="B12" s="45" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="C12" s="45" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="D12" s="51" t="s">
         <v>19</v>
@@ -6144,18 +6187,18 @@
         <v/>
       </c>
       <c r="AX12" s="49" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
     </row>
     <row r="13" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A13" s="45" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="B13" s="45" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="C13" s="45" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="D13" s="50" t="s">
         <v>17</v>
@@ -6335,18 +6378,18 @@
         <v/>
       </c>
       <c r="AX13" s="49" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
     </row>
     <row r="14" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A14" s="45" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="B14" s="45" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="C14" s="45" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="D14" s="51" t="s">
         <v>19</v>
@@ -6526,15 +6569,15 @@
         <v/>
       </c>
       <c r="AX14" s="49" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
     </row>
     <row r="15" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A15" s="23" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="B15" s="24" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="C15" s="24" t="s">
         <v>30</v>
@@ -6597,13 +6640,13 @@
     </row>
     <row r="16" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A16" s="45" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="B16" s="45" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="C16" s="45" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="D16" s="50" t="s">
         <v>17</v>
@@ -6622,21 +6665,21 @@
         <f>WORKDAY(H16,E16-1,Holidays!$A$2:$A$40)</f>
         <v>46304</v>
       </c>
-      <c r="J16" s="47" t="str">
+      <c r="J16" s="47">
         <f>IF('Project Status'!E16="","",'Project Status'!E16)</f>
-        <v/>
-      </c>
-      <c r="K16" s="47" t="str">
+        <v>46304</v>
+      </c>
+      <c r="K16" s="47">
         <f>IF('Project Status'!F16="","",'Project Status'!F16)</f>
-        <v/>
+        <v>46304</v>
       </c>
       <c r="L16" s="45" t="str">
         <f>IF('Project Status'!G16="","",'Project Status'!G16)</f>
-        <v>Pending</v>
-      </c>
-      <c r="M16" s="45" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="M16" s="45">
         <f>IF(OR(K16="",I16=""),"",IF(K16&gt;=I16,NETWORKDAYS(I16,K16,Holidays!$A$2:$A$40)-1,-(NETWORKDAYS(K16,I16,Holidays!$A$2:$A$40)-1)))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N16" s="48" t="str">
         <f t="shared" ref="N16:W24" ca="1" si="4">IF(AND($J16&lt;&gt;"",N$4&gt;=$J16,N$4&lt;=IF($K16="",TODAY(),$K16),N$65=0),"●","")</f>
@@ -6704,7 +6747,7 @@
       </c>
       <c r="AD16" s="48" t="str">
         <f t="shared" ca="1" si="5"/>
-        <v/>
+        <v>●</v>
       </c>
       <c r="AE16" s="48" t="str">
         <f t="shared" ca="1" si="5"/>
@@ -6783,18 +6826,18 @@
         <v/>
       </c>
       <c r="AX16" s="49" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
     </row>
     <row r="17" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A17" s="45" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="B17" s="45" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="C17" s="45" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="D17" s="52" t="s">
         <v>23</v>
@@ -6806,7 +6849,7 @@
         <v>1</v>
       </c>
       <c r="G17" s="45" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="H17" s="47">
         <v>46304</v>
@@ -6815,9 +6858,9 @@
         <f>WORKDAY(H17,E17-1,Holidays!$A$2:$A$40)</f>
         <v>46304</v>
       </c>
-      <c r="J17" s="47" t="str">
+      <c r="J17" s="47">
         <f>IF('Project Status'!E17="","",'Project Status'!E17)</f>
-        <v/>
+        <v>46303</v>
       </c>
       <c r="K17" s="47" t="str">
         <f>IF('Project Status'!F17="","",'Project Status'!F17)</f>
@@ -6825,7 +6868,7 @@
       </c>
       <c r="L17" s="45" t="str">
         <f>IF('Project Status'!G17="","",'Project Status'!G17)</f>
-        <v>Pending</v>
+        <v>In progress</v>
       </c>
       <c r="M17" s="45" t="str">
         <f>IF(OR(K17="",I17=""),"",IF(K17&gt;=I17,NETWORKDAYS(I17,K17,Holidays!$A$2:$A$40)-1,-(NETWORKDAYS(K17,I17,Holidays!$A$2:$A$40)-1)))</f>
@@ -6893,11 +6936,11 @@
       </c>
       <c r="AC17" s="48" t="str">
         <f t="shared" ca="1" si="5"/>
-        <v/>
+        <v>●</v>
       </c>
       <c r="AD17" s="48" t="str">
         <f t="shared" ca="1" si="5"/>
-        <v/>
+        <v>●</v>
       </c>
       <c r="AE17" s="48" t="str">
         <f t="shared" ca="1" si="5"/>
@@ -6976,21 +7019,21 @@
         <v/>
       </c>
       <c r="AX17" s="49" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
     </row>
     <row r="18" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A18" s="45" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="B18" s="45" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="C18" s="45" t="s">
-        <v>159</v>
-      </c>
-      <c r="D18" s="46" t="s">
-        <v>13</v>
+        <v>164</v>
+      </c>
+      <c r="D18" s="54" t="s">
+        <v>37</v>
       </c>
       <c r="E18" s="45">
         <v>1</v>
@@ -6999,7 +7042,7 @@
         <v>1</v>
       </c>
       <c r="G18" s="45" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="H18" s="47">
         <v>46304</v>
@@ -7008,21 +7051,21 @@
         <f>WORKDAY(H18,E18-1,Holidays!$A$2:$A$40)</f>
         <v>46304</v>
       </c>
-      <c r="J18" s="47" t="str">
+      <c r="J18" s="47">
         <f>IF('Project Status'!E18="","",'Project Status'!E18)</f>
-        <v/>
-      </c>
-      <c r="K18" s="47" t="str">
+        <v>46303</v>
+      </c>
+      <c r="K18" s="47">
         <f>IF('Project Status'!F18="","",'Project Status'!F18)</f>
-        <v/>
+        <v>46303</v>
       </c>
       <c r="L18" s="45" t="str">
         <f>IF('Project Status'!G18="","",'Project Status'!G18)</f>
-        <v>Pending</v>
-      </c>
-      <c r="M18" s="45" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="M18" s="45">
         <f>IF(OR(K18="",I18=""),"",IF(K18&gt;=I18,NETWORKDAYS(I18,K18,Holidays!$A$2:$A$40)-1,-(NETWORKDAYS(K18,I18,Holidays!$A$2:$A$40)-1)))</f>
-        <v/>
+        <v>-1</v>
       </c>
       <c r="N18" s="48" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -7086,7 +7129,7 @@
       </c>
       <c r="AC18" s="48" t="str">
         <f t="shared" ca="1" si="5"/>
-        <v/>
+        <v>●</v>
       </c>
       <c r="AD18" s="48" t="str">
         <f t="shared" ca="1" si="5"/>
@@ -7169,21 +7212,21 @@
         <v/>
       </c>
       <c r="AX18" s="49" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
     </row>
     <row r="19" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A19" s="45" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="B19" s="45" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="C19" s="45" t="s">
-        <v>162</v>
-      </c>
-      <c r="D19" s="54" t="s">
-        <v>36</v>
+        <v>167</v>
+      </c>
+      <c r="D19" s="55" t="s">
+        <v>40</v>
       </c>
       <c r="E19" s="45">
         <v>1</v>
@@ -7192,7 +7235,7 @@
         <v>1</v>
       </c>
       <c r="G19" s="45" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="H19" s="47">
         <v>46304</v>
@@ -7201,21 +7244,21 @@
         <f>WORKDAY(H19,E19-1,Holidays!$A$2:$A$40)</f>
         <v>46304</v>
       </c>
-      <c r="J19" s="47" t="str">
+      <c r="J19" s="47">
         <f>IF('Project Status'!E19="","",'Project Status'!E19)</f>
-        <v/>
-      </c>
-      <c r="K19" s="47" t="str">
+        <v>46303</v>
+      </c>
+      <c r="K19" s="47">
         <f>IF('Project Status'!F19="","",'Project Status'!F19)</f>
-        <v/>
+        <v>46303</v>
       </c>
       <c r="L19" s="45" t="str">
         <f>IF('Project Status'!G19="","",'Project Status'!G19)</f>
-        <v>Pending</v>
-      </c>
-      <c r="M19" s="45" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="M19" s="45">
         <f>IF(OR(K19="",I19=""),"",IF(K19&gt;=I19,NETWORKDAYS(I19,K19,Holidays!$A$2:$A$40)-1,-(NETWORKDAYS(K19,I19,Holidays!$A$2:$A$40)-1)))</f>
-        <v/>
+        <v>-1</v>
       </c>
       <c r="N19" s="48" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -7279,7 +7322,7 @@
       </c>
       <c r="AC19" s="48" t="str">
         <f t="shared" ca="1" si="5"/>
-        <v/>
+        <v>●</v>
       </c>
       <c r="AD19" s="48" t="str">
         <f t="shared" ca="1" si="5"/>
@@ -7362,21 +7405,21 @@
         <v/>
       </c>
       <c r="AX19" s="49" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
     </row>
     <row r="20" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A20" s="45" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="B20" s="45" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="C20" s="45" t="s">
-        <v>165</v>
-      </c>
-      <c r="D20" s="55" t="s">
-        <v>38</v>
+        <v>170</v>
+      </c>
+      <c r="D20" s="46" t="s">
+        <v>13</v>
       </c>
       <c r="E20" s="45">
         <v>1</v>
@@ -7385,7 +7428,7 @@
         <v>1</v>
       </c>
       <c r="G20" s="45" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="H20" s="47">
         <v>46304</v>
@@ -7394,21 +7437,21 @@
         <f>WORKDAY(H20,E20-1,Holidays!$A$2:$A$40)</f>
         <v>46304</v>
       </c>
-      <c r="J20" s="47" t="str">
+      <c r="J20" s="47">
         <f>IF('Project Status'!E20="","",'Project Status'!E20)</f>
-        <v/>
-      </c>
-      <c r="K20" s="47" t="str">
+        <v>46303</v>
+      </c>
+      <c r="K20" s="47">
         <f>IF('Project Status'!F20="","",'Project Status'!F20)</f>
-        <v/>
+        <v>46304</v>
       </c>
       <c r="L20" s="45" t="str">
         <f>IF('Project Status'!G20="","",'Project Status'!G20)</f>
-        <v>Pending</v>
-      </c>
-      <c r="M20" s="45" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="M20" s="45">
         <f>IF(OR(K20="",I20=""),"",IF(K20&gt;=I20,NETWORKDAYS(I20,K20,Holidays!$A$2:$A$40)-1,-(NETWORKDAYS(K20,I20,Holidays!$A$2:$A$40)-1)))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N20" s="48" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -7472,11 +7515,11 @@
       </c>
       <c r="AC20" s="48" t="str">
         <f t="shared" ca="1" si="5"/>
-        <v/>
+        <v>●</v>
       </c>
       <c r="AD20" s="48" t="str">
         <f t="shared" ca="1" si="5"/>
-        <v/>
+        <v>●</v>
       </c>
       <c r="AE20" s="48" t="str">
         <f t="shared" ca="1" si="5"/>
@@ -7555,18 +7598,18 @@
         <v/>
       </c>
       <c r="AX20" s="49" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
     </row>
     <row r="21" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A21" s="45" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="B21" s="45" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="C21" s="45" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="D21" s="50" t="s">
         <v>17</v>
@@ -7578,7 +7621,7 @@
         <v>1</v>
       </c>
       <c r="G21" s="45" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="H21" s="47">
         <v>46308</v>
@@ -7748,18 +7791,18 @@
         <v/>
       </c>
       <c r="AX21" s="49" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
     </row>
     <row r="22" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A22" s="45" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="B22" s="45" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="C22" s="45" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="D22" s="50" t="s">
         <v>17</v>
@@ -7771,7 +7814,7 @@
         <v>2</v>
       </c>
       <c r="G22" s="45" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="H22" s="47">
         <v>46311</v>
@@ -7941,18 +7984,18 @@
         <v/>
       </c>
       <c r="AX22" s="49" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
     </row>
     <row r="23" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A23" s="45" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="B23" s="45" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="C23" s="45" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="D23" s="50" t="s">
         <v>17</v>
@@ -7964,7 +8007,7 @@
         <v>1</v>
       </c>
       <c r="G23" s="45" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="H23" s="47">
         <v>46315</v>
@@ -8134,18 +8177,18 @@
         <v/>
       </c>
       <c r="AX23" s="49" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
     </row>
     <row r="24" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A24" s="45" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="B24" s="45" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="C24" s="45" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="D24" s="50" t="s">
         <v>17</v>
@@ -8157,7 +8200,7 @@
         <v>1</v>
       </c>
       <c r="G24" s="45" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="H24" s="47">
         <v>46322</v>
@@ -8327,18 +8370,18 @@
         <v/>
       </c>
       <c r="AX24" s="49" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
     </row>
     <row r="25" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A25" s="27" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="B25" s="28" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="C25" s="28" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="D25" s="28"/>
       <c r="E25" s="28">
@@ -8398,16 +8441,16 @@
     </row>
     <row r="26" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A26" s="45" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="B26" s="45" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="C26" s="45" t="s">
-        <v>182</v>
-      </c>
-      <c r="D26" s="46" t="s">
-        <v>13</v>
+        <v>187</v>
+      </c>
+      <c r="D26" s="54" t="s">
+        <v>37</v>
       </c>
       <c r="E26" s="45">
         <v>1</v>
@@ -8416,7 +8459,7 @@
         <v>1</v>
       </c>
       <c r="G26" s="45" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="H26" s="47">
         <v>46308</v>
@@ -8586,21 +8629,21 @@
         <v/>
       </c>
       <c r="AX26" s="49" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
     </row>
     <row r="27" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A27" s="45" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="B27" s="45" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="C27" s="45" t="s">
-        <v>185</v>
-      </c>
-      <c r="D27" s="55" t="s">
-        <v>38</v>
+        <v>190</v>
+      </c>
+      <c r="D27" s="46" t="s">
+        <v>13</v>
       </c>
       <c r="E27" s="45">
         <v>1</v>
@@ -8609,7 +8652,7 @@
         <v>1</v>
       </c>
       <c r="G27" s="45" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="H27" s="47">
         <v>46308</v>
@@ -8779,21 +8822,21 @@
         <v/>
       </c>
       <c r="AX27" s="49" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
     </row>
     <row r="28" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A28" s="45" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="B28" s="45" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="C28" s="45" t="s">
-        <v>188</v>
-      </c>
-      <c r="D28" s="55" t="s">
-        <v>38</v>
+        <v>193</v>
+      </c>
+      <c r="D28" s="46" t="s">
+        <v>13</v>
       </c>
       <c r="E28" s="45">
         <v>2</v>
@@ -8802,7 +8845,7 @@
         <v>2</v>
       </c>
       <c r="G28" s="45" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="H28" s="47">
         <v>46310</v>
@@ -8972,18 +9015,18 @@
         <v/>
       </c>
       <c r="AX28" s="49" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
     </row>
     <row r="29" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A29" s="45" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="B29" s="45" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="C29" s="45" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
       <c r="D29" s="52" t="s">
         <v>23</v>
@@ -8995,7 +9038,7 @@
         <v>3</v>
       </c>
       <c r="G29" s="45" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="H29" s="47">
         <v>46308</v>
@@ -9165,21 +9208,21 @@
         <v/>
       </c>
       <c r="AX29" s="49" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
     </row>
     <row r="30" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A30" s="45" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="B30" s="45" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="C30" s="45" t="s">
-        <v>195</v>
-      </c>
-      <c r="D30" s="55" t="s">
-        <v>38</v>
+        <v>200</v>
+      </c>
+      <c r="D30" s="46" t="s">
+        <v>13</v>
       </c>
       <c r="E30" s="45">
         <v>1</v>
@@ -9188,7 +9231,7 @@
         <v>1</v>
       </c>
       <c r="G30" s="45" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="H30" s="47">
         <v>46309</v>
@@ -9358,21 +9401,21 @@
         <v/>
       </c>
       <c r="AX30" s="49" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
     </row>
     <row r="31" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A31" s="45" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="B31" s="45" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="C31" s="45" t="s">
-        <v>198</v>
-      </c>
-      <c r="D31" s="54" t="s">
-        <v>36</v>
+        <v>203</v>
+      </c>
+      <c r="D31" s="55" t="s">
+        <v>40</v>
       </c>
       <c r="E31" s="45">
         <v>1</v>
@@ -9381,7 +9424,7 @@
         <v>1</v>
       </c>
       <c r="G31" s="45" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="H31" s="47">
         <v>46308</v>
@@ -9551,21 +9594,21 @@
         <v/>
       </c>
       <c r="AX31" s="49" t="s">
-        <v>199</v>
+        <v>204</v>
       </c>
     </row>
     <row r="32" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A32" s="45" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="B32" s="45" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="C32" s="45" t="s">
-        <v>201</v>
-      </c>
-      <c r="D32" s="55" t="s">
-        <v>38</v>
+        <v>206</v>
+      </c>
+      <c r="D32" s="46" t="s">
+        <v>13</v>
       </c>
       <c r="E32" s="45">
         <v>1</v>
@@ -9574,7 +9617,7 @@
         <v>1</v>
       </c>
       <c r="G32" s="45" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="H32" s="47">
         <v>46314</v>
@@ -9744,18 +9787,18 @@
         <v/>
       </c>
       <c r="AX32" s="49" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
     </row>
     <row r="33" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A33" s="45" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="B33" s="45" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="C33" s="45" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="D33" s="50" t="s">
         <v>17</v>
@@ -9767,7 +9810,7 @@
         <v>1</v>
       </c>
       <c r="G33" s="45" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="H33" s="47">
         <v>46309</v>
@@ -9937,18 +9980,18 @@
         <v/>
       </c>
       <c r="AX33" s="49" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
     </row>
     <row r="34" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A34" s="29" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="B34" s="30" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="C34" s="30" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="D34" s="30"/>
       <c r="E34" s="30">
@@ -10008,16 +10051,16 @@
     </row>
     <row r="35" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A35" s="45" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="B35" s="45" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="C35" s="45" t="s">
-        <v>209</v>
-      </c>
-      <c r="D35" s="46" t="s">
-        <v>13</v>
+        <v>214</v>
+      </c>
+      <c r="D35" s="54" t="s">
+        <v>37</v>
       </c>
       <c r="E35" s="45">
         <v>1</v>
@@ -10026,7 +10069,7 @@
         <v>1</v>
       </c>
       <c r="G35" s="45" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="H35" s="47">
         <v>46310</v>
@@ -10196,21 +10239,21 @@
         <v/>
       </c>
       <c r="AX35" s="49" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
     </row>
     <row r="36" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A36" s="45" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="B36" s="45" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="C36" s="45" t="s">
-        <v>212</v>
-      </c>
-      <c r="D36" s="46" t="s">
-        <v>13</v>
+        <v>217</v>
+      </c>
+      <c r="D36" s="54" t="s">
+        <v>37</v>
       </c>
       <c r="E36" s="45">
         <v>2</v>
@@ -10219,7 +10262,7 @@
         <v>2</v>
       </c>
       <c r="G36" s="45" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="H36" s="47">
         <v>46311</v>
@@ -10389,21 +10432,21 @@
         <v/>
       </c>
       <c r="AX36" s="49" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
     </row>
     <row r="37" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A37" s="45" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
       <c r="B37" s="45" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="C37" s="45" t="s">
-        <v>215</v>
-      </c>
-      <c r="D37" s="54" t="s">
-        <v>36</v>
+        <v>220</v>
+      </c>
+      <c r="D37" s="55" t="s">
+        <v>40</v>
       </c>
       <c r="E37" s="45">
         <v>2</v>
@@ -10412,7 +10455,7 @@
         <v>2</v>
       </c>
       <c r="G37" s="45" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="H37" s="47">
         <v>46309</v>
@@ -10582,21 +10625,21 @@
         <v/>
       </c>
       <c r="AX37" s="49" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
     </row>
     <row r="38" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A38" s="45" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="B38" s="45" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="C38" s="45" t="s">
-        <v>219</v>
-      </c>
-      <c r="D38" s="54" t="s">
-        <v>36</v>
+        <v>224</v>
+      </c>
+      <c r="D38" s="55" t="s">
+        <v>40</v>
       </c>
       <c r="E38" s="45">
         <v>2</v>
@@ -10605,7 +10648,7 @@
         <v>2</v>
       </c>
       <c r="G38" s="45" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
       <c r="H38" s="47">
         <v>46311</v>
@@ -10775,21 +10818,21 @@
         <v/>
       </c>
       <c r="AX38" s="49" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
     </row>
     <row r="39" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A39" s="45" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B39" s="45" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="C39" s="45" t="s">
-        <v>222</v>
-      </c>
-      <c r="D39" s="54" t="s">
-        <v>36</v>
+        <v>227</v>
+      </c>
+      <c r="D39" s="55" t="s">
+        <v>40</v>
       </c>
       <c r="E39" s="45">
         <v>1</v>
@@ -10798,7 +10841,7 @@
         <v>1</v>
       </c>
       <c r="G39" s="45" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="H39" s="47">
         <v>46315</v>
@@ -10968,18 +11011,18 @@
         <v/>
       </c>
       <c r="AX39" s="49" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
     </row>
     <row r="40" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A40" s="45" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="B40" s="45" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="C40" s="45" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="D40" s="52" t="s">
         <v>23</v>
@@ -10991,7 +11034,7 @@
         <v>1</v>
       </c>
       <c r="G40" s="45" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="H40" s="47">
         <v>46314</v>
@@ -11161,18 +11204,18 @@
         <v/>
       </c>
       <c r="AX40" s="49" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
     </row>
     <row r="41" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A41" s="45" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="B41" s="45" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="C41" s="45" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="D41" s="52" t="s">
         <v>23</v>
@@ -11184,7 +11227,7 @@
         <v>1</v>
       </c>
       <c r="G41" s="45" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="H41" s="47">
         <v>46315</v>
@@ -11354,18 +11397,18 @@
         <v/>
       </c>
       <c r="AX41" s="49" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
     </row>
     <row r="42" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A42" s="45" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="B42" s="45" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="C42" s="45" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="D42" s="50" t="s">
         <v>17</v>
@@ -11377,7 +11420,7 @@
         <v>1</v>
       </c>
       <c r="G42" s="45" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="H42" s="47">
         <v>46316</v>
@@ -11547,21 +11590,21 @@
         <v/>
       </c>
       <c r="AX42" s="49" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
     </row>
     <row r="43" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A43" s="45" t="s">
-        <v>236</v>
+        <v>241</v>
       </c>
       <c r="B43" s="45" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="C43" s="45" t="s">
-        <v>237</v>
-      </c>
-      <c r="D43" s="55" t="s">
-        <v>38</v>
+        <v>242</v>
+      </c>
+      <c r="D43" s="46" t="s">
+        <v>13</v>
       </c>
       <c r="E43" s="45">
         <v>1</v>
@@ -11570,7 +11613,7 @@
         <v>1</v>
       </c>
       <c r="G43" s="45" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="H43" s="47">
         <v>46315</v>
@@ -11740,18 +11783,18 @@
         <v/>
       </c>
       <c r="AX43" s="49" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
     </row>
     <row r="44" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A44" s="31" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="B44" s="32" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="C44" s="32" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="D44" s="32"/>
       <c r="E44" s="32">
@@ -11811,13 +11854,13 @@
     </row>
     <row r="45" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A45" s="45" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="B45" s="45" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="C45" s="45" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="D45" s="52" t="s">
         <v>23</v>
@@ -11829,7 +11872,7 @@
         <v>2</v>
       </c>
       <c r="G45" s="45" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="H45" s="47">
         <v>46316</v>
@@ -11999,21 +12042,21 @@
         <v/>
       </c>
       <c r="AX45" s="49" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
     </row>
     <row r="46" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A46" s="45" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="B46" s="45" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="C46" s="45" t="s">
-        <v>244</v>
-      </c>
-      <c r="D46" s="55" t="s">
-        <v>38</v>
+        <v>249</v>
+      </c>
+      <c r="D46" s="46" t="s">
+        <v>13</v>
       </c>
       <c r="E46" s="45">
         <v>2</v>
@@ -12022,7 +12065,7 @@
         <v>2</v>
       </c>
       <c r="G46" s="45" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="H46" s="47">
         <v>46316</v>
@@ -12192,21 +12235,21 @@
         <v/>
       </c>
       <c r="AX46" s="49" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
     </row>
     <row r="47" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A47" s="45" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="B47" s="45" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="C47" s="45" t="s">
-        <v>248</v>
-      </c>
-      <c r="D47" s="46" t="s">
-        <v>13</v>
+        <v>253</v>
+      </c>
+      <c r="D47" s="54" t="s">
+        <v>37</v>
       </c>
       <c r="E47" s="45">
         <v>2</v>
@@ -12215,7 +12258,7 @@
         <v>2</v>
       </c>
       <c r="G47" s="45" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="H47" s="47">
         <v>46315</v>
@@ -12385,21 +12428,21 @@
         <v/>
       </c>
       <c r="AX47" s="49" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
     </row>
     <row r="48" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A48" s="45" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="B48" s="45" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="C48" s="45" t="s">
-        <v>251</v>
-      </c>
-      <c r="D48" s="54" t="s">
-        <v>36</v>
+        <v>256</v>
+      </c>
+      <c r="D48" s="55" t="s">
+        <v>40</v>
       </c>
       <c r="E48" s="45">
         <v>2</v>
@@ -12408,7 +12451,7 @@
         <v>2</v>
       </c>
       <c r="G48" s="45" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="H48" s="47">
         <v>46316</v>
@@ -12578,18 +12621,18 @@
         <v/>
       </c>
       <c r="AX48" s="49" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
     </row>
     <row r="49" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A49" s="45" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="B49" s="45" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="C49" s="45" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="D49" s="50" t="s">
         <v>17</v>
@@ -12601,7 +12644,7 @@
         <v>2</v>
       </c>
       <c r="G49" s="45" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="H49" s="47">
         <v>46317</v>
@@ -12771,18 +12814,18 @@
         <v/>
       </c>
       <c r="AX49" s="49" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
     </row>
     <row r="50" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A50" s="45" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="B50" s="45" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="C50" s="45" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="D50" s="52" t="s">
         <v>23</v>
@@ -12794,7 +12837,7 @@
         <v>1</v>
       </c>
       <c r="G50" s="45" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
       <c r="H50" s="47">
         <v>46321</v>
@@ -12964,21 +13007,21 @@
         <v/>
       </c>
       <c r="AX50" s="49" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
     </row>
     <row r="51" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A51" s="45" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="B51" s="45" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="C51" s="45" t="s">
-        <v>260</v>
-      </c>
-      <c r="D51" s="46" t="s">
-        <v>13</v>
+        <v>265</v>
+      </c>
+      <c r="D51" s="54" t="s">
+        <v>37</v>
       </c>
       <c r="E51" s="45">
         <v>1</v>
@@ -12987,7 +13030,7 @@
         <v>1</v>
       </c>
       <c r="G51" s="45" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="H51" s="47">
         <v>46322</v>
@@ -13157,21 +13200,21 @@
         <v/>
       </c>
       <c r="AX51" s="49" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
     </row>
     <row r="52" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A52" s="45" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="B52" s="45" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="C52" s="45" t="s">
-        <v>263</v>
-      </c>
-      <c r="D52" s="55" t="s">
-        <v>38</v>
+        <v>268</v>
+      </c>
+      <c r="D52" s="46" t="s">
+        <v>13</v>
       </c>
       <c r="E52" s="45">
         <v>1</v>
@@ -13180,7 +13223,7 @@
         <v>1</v>
       </c>
       <c r="G52" s="45" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="H52" s="47">
         <v>46322</v>
@@ -13350,18 +13393,18 @@
         <v/>
       </c>
       <c r="AX52" s="49" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
     </row>
     <row r="53" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A53" s="45" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="B53" s="45" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="C53" s="45" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="D53" s="52" t="s">
         <v>23</v>
@@ -13373,7 +13416,7 @@
         <v>1</v>
       </c>
       <c r="G53" s="45" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="H53" s="47">
         <v>46323</v>
@@ -13543,18 +13586,18 @@
         <v/>
       </c>
       <c r="AX53" s="49" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
     </row>
     <row r="54" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A54" s="45" t="s">
-        <v>269</v>
+        <v>274</v>
       </c>
       <c r="B54" s="45" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="C54" s="45" t="s">
-        <v>270</v>
+        <v>275</v>
       </c>
       <c r="D54" s="52" t="s">
         <v>23</v>
@@ -13566,7 +13609,7 @@
         <v>1</v>
       </c>
       <c r="G54" s="45" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="H54" s="47">
         <v>46324</v>
@@ -13736,21 +13779,21 @@
         <v/>
       </c>
       <c r="AX54" s="49" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
     </row>
     <row r="55" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A55" s="45" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="B55" s="45" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="C55" s="45" t="s">
-        <v>273</v>
-      </c>
-      <c r="D55" s="55" t="s">
-        <v>38</v>
+        <v>278</v>
+      </c>
+      <c r="D55" s="46" t="s">
+        <v>13</v>
       </c>
       <c r="E55" s="45">
         <v>1</v>
@@ -13759,7 +13802,7 @@
         <v>1</v>
       </c>
       <c r="G55" s="45" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="H55" s="47">
         <v>46324</v>
@@ -13929,18 +13972,18 @@
         <v/>
       </c>
       <c r="AX55" s="49" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
     </row>
     <row r="56" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A56" s="45" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="B56" s="45" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="C56" s="45" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="D56" s="50" t="s">
         <v>17</v>
@@ -13952,7 +13995,7 @@
         <v>1</v>
       </c>
       <c r="G56" s="45" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="H56" s="47">
         <v>46324</v>
@@ -14122,21 +14165,21 @@
         <v/>
       </c>
       <c r="AX56" s="49" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
     </row>
     <row r="57" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A57" s="45" t="s">
-        <v>278</v>
+        <v>283</v>
       </c>
       <c r="B57" s="45" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="C57" s="45" t="s">
-        <v>279</v>
-      </c>
-      <c r="D57" s="46" t="s">
-        <v>13</v>
+        <v>284</v>
+      </c>
+      <c r="D57" s="54" t="s">
+        <v>37</v>
       </c>
       <c r="E57" s="45">
         <v>1</v>
@@ -14145,7 +14188,7 @@
         <v>1</v>
       </c>
       <c r="G57" s="45" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="H57" s="47">
         <v>46324</v>
@@ -14315,21 +14358,21 @@
         <v/>
       </c>
       <c r="AX57" s="49" t="s">
-        <v>280</v>
+        <v>285</v>
       </c>
     </row>
     <row r="58" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A58" s="45" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="B58" s="45" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="C58" s="45" t="s">
-        <v>282</v>
-      </c>
-      <c r="D58" s="54" t="s">
-        <v>36</v>
+        <v>287</v>
+      </c>
+      <c r="D58" s="55" t="s">
+        <v>40</v>
       </c>
       <c r="E58" s="45">
         <v>1</v>
@@ -14338,7 +14381,7 @@
         <v>1</v>
       </c>
       <c r="G58" s="45" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="H58" s="47">
         <v>46324</v>
@@ -14508,21 +14551,21 @@
         <v/>
       </c>
       <c r="AX58" s="49" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
     </row>
     <row r="59" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A59" s="45" t="s">
-        <v>284</v>
+        <v>289</v>
       </c>
       <c r="B59" s="45" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="C59" s="45" t="s">
-        <v>285</v>
-      </c>
-      <c r="D59" s="55" t="s">
-        <v>38</v>
+        <v>290</v>
+      </c>
+      <c r="D59" s="46" t="s">
+        <v>13</v>
       </c>
       <c r="E59" s="45">
         <v>1</v>
@@ -14531,7 +14574,7 @@
         <v>1</v>
       </c>
       <c r="G59" s="45" t="s">
-        <v>286</v>
+        <v>291</v>
       </c>
       <c r="H59" s="47">
         <v>46325</v>
@@ -14701,21 +14744,21 @@
         <v/>
       </c>
       <c r="AX59" s="49" t="s">
-        <v>287</v>
+        <v>292</v>
       </c>
     </row>
     <row r="60" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A60" s="45" t="s">
-        <v>288</v>
+        <v>293</v>
       </c>
       <c r="B60" s="45" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="C60" s="45" t="s">
-        <v>289</v>
-      </c>
-      <c r="D60" s="46" t="s">
-        <v>13</v>
+        <v>294</v>
+      </c>
+      <c r="D60" s="54" t="s">
+        <v>37</v>
       </c>
       <c r="E60" s="45">
         <v>2</v>
@@ -14724,7 +14767,7 @@
         <v>2</v>
       </c>
       <c r="G60" s="45" t="s">
-        <v>284</v>
+        <v>289</v>
       </c>
       <c r="H60" s="47">
         <v>46328</v>
@@ -14894,84 +14937,84 @@
         <v/>
       </c>
       <c r="AX60" s="49" t="s">
-        <v>290</v>
+        <v>295</v>
       </c>
     </row>
     <row r="62" spans="1:50" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C62" s="59" t="s">
-        <v>291</v>
+        <v>296</v>
       </c>
       <c r="N62" s="60" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
       <c r="AD62" s="60" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="AJ62" s="60" t="s">
-        <v>294</v>
+        <v>299</v>
       </c>
       <c r="AL62" s="60" t="s">
-        <v>295</v>
+        <v>300</v>
       </c>
       <c r="AM62" s="60" t="s">
-        <v>296</v>
+        <v>301</v>
       </c>
       <c r="AO62" s="60" t="s">
-        <v>297</v>
+        <v>302</v>
       </c>
       <c r="AQ62" s="60" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="AW62" s="60" t="s">
-        <v>299</v>
+        <v>304</v>
       </c>
     </row>
     <row r="63" spans="1:50" x14ac:dyDescent="0.2">
       <c r="C63" s="33" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="N63" s="61" t="s">
-        <v>301</v>
+        <v>306</v>
       </c>
       <c r="P63" s="61" t="s">
-        <v>302</v>
+        <v>307</v>
       </c>
       <c r="U63" s="61" t="s">
-        <v>303</v>
+        <v>308</v>
       </c>
       <c r="X63" s="61" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
       <c r="Z63" s="61" t="s">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="AC63" s="61" t="s">
-        <v>306</v>
+        <v>311</v>
       </c>
       <c r="AH63" s="61" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="AJ63" s="61" t="s">
-        <v>308</v>
+        <v>313</v>
       </c>
       <c r="AM63" s="61" t="s">
-        <v>309</v>
+        <v>314</v>
       </c>
       <c r="AO63" s="61" t="s">
-        <v>310</v>
+        <v>315</v>
       </c>
       <c r="AW63" s="61" t="s">
-        <v>311</v>
+        <v>316</v>
       </c>
     </row>
     <row r="64" spans="1:50" x14ac:dyDescent="0.2">
       <c r="C64" s="62" t="s">
-        <v>312</v>
+        <v>317</v>
       </c>
     </row>
     <row r="65" spans="3:49" hidden="1" x14ac:dyDescent="0.2">
       <c r="C65" t="s">
-        <v>313</v>
+        <v>318</v>
       </c>
       <c r="N65">
         <f>IF(COUNTIF(Holidays!$A$2:$A$40,N$4)&gt;0,1,0)</f>
@@ -15304,33 +15347,33 @@
   <sheetData>
     <row r="1" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="63" t="s">
-        <v>314</v>
+        <v>319</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="28" x14ac:dyDescent="0.2">
       <c r="A3" s="11" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>315</v>
+        <v>320</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>316</v>
+        <v>321</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>317</v>
+        <v>322</v>
       </c>
       <c r="E3" s="11" t="s">
-        <v>318</v>
+        <v>323</v>
       </c>
       <c r="F3" s="11" t="s">
         <v>14</v>
       </c>
       <c r="G3" s="11" t="s">
-        <v>85</v>
+        <v>34</v>
       </c>
       <c r="H3" s="11" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
@@ -15338,10 +15381,10 @@
         <v>23</v>
       </c>
       <c r="B4" s="65" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="C4" s="65" t="s">
-        <v>321</v>
+        <v>326</v>
       </c>
       <c r="D4" s="65">
         <f>COUNTIFS(Tasks!$D$5:$D$60,A4,Tasks!$B$5:$B$60,"&lt;&gt;P0",Tasks!$A$5:$A$60,"&lt;&gt;WP*")</f>
@@ -15357,7 +15400,7 @@
       </c>
       <c r="G4" s="65">
         <f>COUNTIFS(Tasks!$D$5:$D$60,A4,Tasks!$L$5:$L$60,"In progress")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H4" s="65">
         <f>COUNTIFS(Tasks!$D$5:$D$60,A4,Tasks!$L$5:$L$60,"Incident")</f>
@@ -15366,25 +15409,25 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" s="66" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B5" s="65" t="s">
-        <v>322</v>
+        <v>327</v>
       </c>
       <c r="C5" s="65" t="s">
-        <v>323</v>
+        <v>328</v>
       </c>
       <c r="D5" s="65">
         <f>COUNTIFS(Tasks!$D$5:$D$60,A5,Tasks!$B$5:$B$60,"&lt;&gt;P0",Tasks!$A$5:$A$60,"&lt;&gt;WP*")</f>
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E5" s="65">
         <f>SUMIFS(Tasks!$F$5:$F$60,Tasks!$D$5:$D$60,A5,Tasks!$B$5:$B$60,"&lt;&gt;P0")</f>
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F5" s="65">
         <f>COUNTIFS(Tasks!$D$5:$D$60,A5,Tasks!$L$5:$L$60,"Completed",Tasks!$B$5:$B$60,"&lt;&gt;P0")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G5" s="65">
         <f>COUNTIFS(Tasks!$D$5:$D$60,A5,Tasks!$L$5:$L$60,"In progress")</f>
@@ -15400,10 +15443,10 @@
         <v>17</v>
       </c>
       <c r="B6" s="65" t="s">
-        <v>324</v>
+        <v>329</v>
       </c>
       <c r="C6" s="65" t="s">
-        <v>325</v>
+        <v>330</v>
       </c>
       <c r="D6" s="65">
         <f>COUNTIFS(Tasks!$D$5:$D$60,A6,Tasks!$B$5:$B$60,"&lt;&gt;P0",Tasks!$A$5:$A$60,"&lt;&gt;WP*")</f>
@@ -15415,7 +15458,7 @@
       </c>
       <c r="F6" s="65">
         <f>COUNTIFS(Tasks!$D$5:$D$60,A6,Tasks!$L$5:$L$60,"Completed",Tasks!$B$5:$B$60,"&lt;&gt;P0")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G6" s="65">
         <f>COUNTIFS(Tasks!$D$5:$D$60,A6,Tasks!$L$5:$L$60,"In progress")</f>
@@ -15431,22 +15474,22 @@
         <v>13</v>
       </c>
       <c r="B7" s="65" t="s">
-        <v>326</v>
+        <v>331</v>
       </c>
       <c r="C7" s="65" t="s">
-        <v>327</v>
+        <v>332</v>
       </c>
       <c r="D7" s="65">
         <f>COUNTIFS(Tasks!$D$5:$D$60,A7,Tasks!$B$5:$B$60,"&lt;&gt;P0",Tasks!$A$5:$A$60,"&lt;&gt;WP*")</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E7" s="65">
         <f>SUMIFS(Tasks!$F$5:$F$60,Tasks!$D$5:$D$60,A7,Tasks!$B$5:$B$60,"&lt;&gt;P0")</f>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F7" s="65">
         <f>COUNTIFS(Tasks!$D$5:$D$60,A7,Tasks!$L$5:$L$60,"Completed",Tasks!$B$5:$B$60,"&lt;&gt;P0")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G7" s="65">
         <f>COUNTIFS(Tasks!$D$5:$D$60,A7,Tasks!$L$5:$L$60,"In progress")</f>
@@ -15459,13 +15502,13 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" s="69" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B8" s="65" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
       <c r="C8" s="65" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
       <c r="D8" s="65">
         <f>COUNTIFS(Tasks!$D$5:$D$60,A8,Tasks!$B$5:$B$60,"&lt;&gt;P0",Tasks!$A$5:$A$60,"&lt;&gt;WP*")</f>
@@ -15477,7 +15520,7 @@
       </c>
       <c r="F8" s="65">
         <f>COUNTIFS(Tasks!$D$5:$D$60,A8,Tasks!$L$5:$L$60,"Completed",Tasks!$B$5:$B$60,"&lt;&gt;P0")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G8" s="65">
         <f>COUNTIFS(Tasks!$D$5:$D$60,A8,Tasks!$L$5:$L$60,"In progress")</f>
@@ -15490,7 +15533,7 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="70" t="s">
-        <v>330</v>
+        <v>335</v>
       </c>
       <c r="D9" s="70">
         <f>SUM(D4:D8)</f>
@@ -15502,11 +15545,11 @@
       </c>
       <c r="F9" s="70">
         <f>SUM(F4:F8)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G9" s="70">
         <f>SUM(G4:G8)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H9" s="70">
         <f>SUM(H4:H8)</f>
@@ -15533,33 +15576,33 @@
   <sheetData>
     <row r="1" spans="1:7" ht="42" x14ac:dyDescent="0.2">
       <c r="A1" s="11" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="B1" s="11" t="s">
-        <v>331</v>
+        <v>336</v>
       </c>
       <c r="C1" s="11" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D1" s="11" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="E1" s="11" t="s">
         <v>9</v>
       </c>
       <c r="F1" s="11" t="s">
-        <v>334</v>
+        <v>339</v>
       </c>
       <c r="G1" s="11" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="65" t="s">
-        <v>335</v>
+        <v>340</v>
       </c>
       <c r="B2" s="65" t="s">
-        <v>336</v>
+        <v>341</v>
       </c>
       <c r="C2" s="71">
         <v>46282</v>
@@ -15571,7 +15614,7 @@
         <v>14</v>
       </c>
       <c r="F2" s="65" t="s">
-        <v>337</v>
+        <v>342</v>
       </c>
       <c r="G2" s="65">
         <f>IF(D2="","",IF(D2&gt;=C2,NETWORKDAYS(C2,D2,Holidays!$A$2:$A$40)-1,-(NETWORKDAYS(D2,C2,Holidays!$A$2:$A$40)-1)))</f>
@@ -15580,20 +15623,20 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="65" t="s">
-        <v>338</v>
+        <v>343</v>
       </c>
       <c r="B3" s="65" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
       <c r="C3" s="71">
         <v>46304</v>
       </c>
       <c r="D3" s="72"/>
       <c r="E3" s="73" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="F3" s="65" t="s">
-        <v>340</v>
+        <v>345</v>
       </c>
       <c r="G3" s="65" t="str">
         <f>IF(D3="","",IF(D3&gt;=C3,NETWORKDAYS(C3,D3,Holidays!$A$2:$A$40)-1,-(NETWORKDAYS(D3,C3,Holidays!$A$2:$A$40)-1)))</f>
@@ -15602,20 +15645,20 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="65" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
       <c r="B4" s="65" t="s">
-        <v>342</v>
+        <v>347</v>
       </c>
       <c r="C4" s="71">
         <v>46314</v>
       </c>
       <c r="D4" s="72"/>
       <c r="E4" s="73" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="F4" s="65" t="s">
-        <v>343</v>
+        <v>348</v>
       </c>
       <c r="G4" s="65" t="str">
         <f>IF(D4="","",IF(D4&gt;=C4,NETWORKDAYS(C4,D4,Holidays!$A$2:$A$40)-1,-(NETWORKDAYS(D4,C4,Holidays!$A$2:$A$40)-1)))</f>
@@ -15624,20 +15667,20 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" s="65" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="B5" s="65" t="s">
-        <v>345</v>
+        <v>350</v>
       </c>
       <c r="C5" s="71">
         <v>46316</v>
       </c>
       <c r="D5" s="72"/>
       <c r="E5" s="73" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="F5" s="65" t="s">
-        <v>346</v>
+        <v>351</v>
       </c>
       <c r="G5" s="65" t="str">
         <f>IF(D5="","",IF(D5&gt;=C5,NETWORKDAYS(C5,D5,Holidays!$A$2:$A$40)-1,-(NETWORKDAYS(D5,C5,Holidays!$A$2:$A$40)-1)))</f>
@@ -15646,20 +15689,20 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="65" t="s">
-        <v>347</v>
+        <v>352</v>
       </c>
       <c r="B6" s="65" t="s">
-        <v>348</v>
+        <v>353</v>
       </c>
       <c r="C6" s="71">
         <v>46317</v>
       </c>
       <c r="D6" s="72"/>
       <c r="E6" s="73" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="F6" s="65" t="s">
-        <v>349</v>
+        <v>354</v>
       </c>
       <c r="G6" s="65" t="str">
         <f>IF(D6="","",IF(D6&gt;=C6,NETWORKDAYS(C6,D6,Holidays!$A$2:$A$40)-1,-(NETWORKDAYS(D6,C6,Holidays!$A$2:$A$40)-1)))</f>
@@ -15668,20 +15711,20 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="65" t="s">
-        <v>350</v>
+        <v>355</v>
       </c>
       <c r="B7" s="65" t="s">
-        <v>351</v>
+        <v>356</v>
       </c>
       <c r="C7" s="71">
         <v>46321</v>
       </c>
       <c r="D7" s="72"/>
       <c r="E7" s="73" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="F7" s="65" t="s">
-        <v>352</v>
+        <v>357</v>
       </c>
       <c r="G7" s="65" t="str">
         <f>IF(D7="","",IF(D7&gt;=C7,NETWORKDAYS(C7,D7,Holidays!$A$2:$A$40)-1,-(NETWORKDAYS(D7,C7,Holidays!$A$2:$A$40)-1)))</f>
@@ -15690,20 +15733,20 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" s="65" t="s">
-        <v>353</v>
+        <v>358</v>
       </c>
       <c r="B8" s="65" t="s">
-        <v>354</v>
+        <v>359</v>
       </c>
       <c r="C8" s="71">
         <v>46323</v>
       </c>
       <c r="D8" s="72"/>
       <c r="E8" s="73" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="F8" s="65" t="s">
-        <v>340</v>
+        <v>345</v>
       </c>
       <c r="G8" s="65" t="str">
         <f>IF(D8="","",IF(D8&gt;=C8,NETWORKDAYS(C8,D8,Holidays!$A$2:$A$40)-1,-(NETWORKDAYS(D8,C8,Holidays!$A$2:$A$40)-1)))</f>
@@ -15712,20 +15755,20 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" s="65" t="s">
-        <v>355</v>
+        <v>360</v>
       </c>
       <c r="B9" s="65" t="s">
-        <v>356</v>
+        <v>361</v>
       </c>
       <c r="C9" s="71">
         <v>46331</v>
       </c>
       <c r="D9" s="72"/>
       <c r="E9" s="73" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="F9" s="65" t="s">
-        <v>357</v>
+        <v>362</v>
       </c>
       <c r="G9" s="65" t="str">
         <f>IF(D9="","",IF(D9&gt;=C9,NETWORKDAYS(C9,D9,Holidays!$A$2:$A$40)-1,-(NETWORKDAYS(D9,C9,Holidays!$A$2:$A$40)-1)))</f>
@@ -15761,39 +15804,39 @@
   <sheetData>
     <row r="1" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="63" t="s">
-        <v>358</v>
+        <v>363</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" s="11" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>359</v>
+        <v>364</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>360</v>
+        <v>365</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>361</v>
+        <v>366</v>
       </c>
       <c r="E3" s="11" t="s">
-        <v>362</v>
+        <v>367</v>
       </c>
       <c r="F3" s="11" t="s">
-        <v>363</v>
+        <v>368</v>
       </c>
       <c r="G3" s="11" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="H3" s="11" t="s">
         <v>9</v>
       </c>
       <c r="I3" s="11" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
       <c r="J3" s="11" t="s">
-        <v>365</v>
+        <v>370</v>
       </c>
       <c r="K3" s="11" t="s">
         <v>10</v>
@@ -15801,10 +15844,10 @@
     </row>
     <row r="4" spans="1:11" ht="28" x14ac:dyDescent="0.2">
       <c r="A4" s="74" t="s">
-        <v>366</v>
+        <v>371</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>367</v>
+        <v>372</v>
       </c>
       <c r="C4" s="75">
         <v>3</v>
@@ -15824,10 +15867,10 @@
         <v>17</v>
       </c>
       <c r="H4" s="75" t="s">
-        <v>368</v>
+        <v>373</v>
       </c>
       <c r="I4" s="14" t="s">
-        <v>369</v>
+        <v>374</v>
       </c>
       <c r="J4" s="76">
         <v>46303</v>
@@ -15836,10 +15879,10 @@
     </row>
     <row r="5" spans="1:11" ht="28" x14ac:dyDescent="0.2">
       <c r="A5" s="74" t="s">
-        <v>370</v>
+        <v>375</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>371</v>
+        <v>376</v>
       </c>
       <c r="C5" s="75">
         <v>3</v>
@@ -15855,14 +15898,14 @@
         <f t="shared" si="1"/>
         <v>High</v>
       </c>
-      <c r="G5" s="25" t="s">
-        <v>36</v>
+      <c r="G5" s="26" t="s">
+        <v>40</v>
       </c>
       <c r="H5" s="75" t="s">
-        <v>368</v>
+        <v>373</v>
       </c>
       <c r="I5" s="14" t="s">
-        <v>372</v>
+        <v>377</v>
       </c>
       <c r="J5" s="76">
         <v>46303</v>
@@ -15871,10 +15914,10 @@
     </row>
     <row r="6" spans="1:11" ht="28" x14ac:dyDescent="0.2">
       <c r="A6" s="74" t="s">
-        <v>373</v>
+        <v>378</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>374</v>
+        <v>379</v>
       </c>
       <c r="C6" s="75">
         <v>1</v>
@@ -15890,14 +15933,14 @@
         <f t="shared" si="1"/>
         <v>Medium</v>
       </c>
-      <c r="G6" s="26" t="s">
-        <v>38</v>
+      <c r="G6" s="25" t="s">
+        <v>37</v>
       </c>
       <c r="H6" s="75" t="s">
-        <v>375</v>
+        <v>380</v>
       </c>
       <c r="I6" s="14" t="s">
-        <v>376</v>
+        <v>381</v>
       </c>
       <c r="J6" s="76">
         <v>46303</v>
@@ -15906,10 +15949,10 @@
     </row>
     <row r="7" spans="1:11" ht="28" x14ac:dyDescent="0.2">
       <c r="A7" s="74" t="s">
-        <v>377</v>
+        <v>382</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>378</v>
+        <v>383</v>
       </c>
       <c r="C7" s="75">
         <v>2</v>
@@ -15929,10 +15972,10 @@
         <v>17</v>
       </c>
       <c r="H7" s="75" t="s">
-        <v>379</v>
+        <v>384</v>
       </c>
       <c r="I7" s="14" t="s">
-        <v>380</v>
+        <v>385</v>
       </c>
       <c r="J7" s="76">
         <v>46303</v>
@@ -15941,10 +15984,10 @@
     </row>
     <row r="8" spans="1:11" ht="28" x14ac:dyDescent="0.2">
       <c r="A8" s="74" t="s">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>382</v>
+        <v>387</v>
       </c>
       <c r="C8" s="75">
         <v>2</v>
@@ -15960,14 +16003,14 @@
         <f t="shared" si="1"/>
         <v>High</v>
       </c>
-      <c r="G8" s="26" t="s">
-        <v>38</v>
+      <c r="G8" s="25" t="s">
+        <v>37</v>
       </c>
       <c r="H8" s="75" t="s">
-        <v>379</v>
+        <v>384</v>
       </c>
       <c r="I8" s="14" t="s">
-        <v>383</v>
+        <v>388</v>
       </c>
       <c r="J8" s="76">
         <v>46303</v>
@@ -15976,10 +16019,10 @@
     </row>
     <row r="9" spans="1:11" ht="28" x14ac:dyDescent="0.2">
       <c r="A9" s="74" t="s">
-        <v>384</v>
+        <v>389</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>385</v>
+        <v>390</v>
       </c>
       <c r="C9" s="75">
         <v>2</v>
@@ -15995,14 +16038,14 @@
         <f t="shared" si="1"/>
         <v>Medium</v>
       </c>
-      <c r="G9" s="25" t="s">
-        <v>36</v>
+      <c r="G9" s="26" t="s">
+        <v>40</v>
       </c>
       <c r="H9" s="75" t="s">
-        <v>379</v>
+        <v>384</v>
       </c>
       <c r="I9" s="14" t="s">
-        <v>386</v>
+        <v>391</v>
       </c>
       <c r="J9" s="76">
         <v>46303</v>
@@ -16011,10 +16054,10 @@
     </row>
     <row r="10" spans="1:11" ht="28" x14ac:dyDescent="0.2">
       <c r="A10" s="74" t="s">
-        <v>387</v>
+        <v>392</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>388</v>
+        <v>393</v>
       </c>
       <c r="C10" s="75">
         <v>1</v>
@@ -16034,10 +16077,10 @@
         <v>13</v>
       </c>
       <c r="H10" s="75" t="s">
-        <v>379</v>
+        <v>384</v>
       </c>
       <c r="I10" s="14" t="s">
-        <v>389</v>
+        <v>394</v>
       </c>
       <c r="J10" s="76">
         <v>46303</v>
@@ -16046,10 +16089,10 @@
     </row>
     <row r="11" spans="1:11" ht="28" x14ac:dyDescent="0.2">
       <c r="A11" s="74" t="s">
-        <v>390</v>
+        <v>395</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>391</v>
+        <v>396</v>
       </c>
       <c r="C11" s="75">
         <v>2</v>
@@ -16069,10 +16112,10 @@
         <v>13</v>
       </c>
       <c r="H11" s="75" t="s">
-        <v>379</v>
+        <v>384</v>
       </c>
       <c r="I11" s="14" t="s">
-        <v>392</v>
+        <v>397</v>
       </c>
       <c r="J11" s="76">
         <v>46303</v>
@@ -16081,10 +16124,10 @@
     </row>
     <row r="12" spans="1:11" ht="28" x14ac:dyDescent="0.2">
       <c r="A12" s="74" t="s">
-        <v>393</v>
+        <v>398</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>394</v>
+        <v>399</v>
       </c>
       <c r="C12" s="75">
         <v>2</v>
@@ -16104,10 +16147,10 @@
         <v>23</v>
       </c>
       <c r="H12" s="75" t="s">
-        <v>379</v>
+        <v>384</v>
       </c>
       <c r="I12" s="14" t="s">
-        <v>395</v>
+        <v>400</v>
       </c>
       <c r="J12" s="76">
         <v>46303</v>
@@ -16116,10 +16159,10 @@
     </row>
     <row r="13" spans="1:11" ht="28" x14ac:dyDescent="0.2">
       <c r="A13" s="74" t="s">
-        <v>396</v>
+        <v>401</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>397</v>
+        <v>402</v>
       </c>
       <c r="C13" s="75">
         <v>2</v>
@@ -16139,10 +16182,10 @@
         <v>23</v>
       </c>
       <c r="H13" s="75" t="s">
-        <v>379</v>
+        <v>384</v>
       </c>
       <c r="I13" s="14" t="s">
-        <v>398</v>
+        <v>403</v>
       </c>
       <c r="J13" s="76">
         <v>46303</v>
@@ -16182,10 +16225,10 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="11" t="s">
-        <v>399</v>
+        <v>404</v>
       </c>
       <c r="B1" s="11" t="s">
-        <v>400</v>
+        <v>405</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
@@ -16193,10 +16236,10 @@
         <v>46289</v>
       </c>
       <c r="B2" s="78" t="s">
-        <v>401</v>
+        <v>406</v>
       </c>
       <c r="D2" s="79" t="s">
-        <v>402</v>
+        <v>407</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
@@ -16204,7 +16247,7 @@
         <v>46307</v>
       </c>
       <c r="B3" s="78" t="s">
-        <v>403</v>
+        <v>408</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Project Status up to 24 Oct
</commit_message>
<xml_diff>
--- a/status/Gantt_live_11DP-C.xlsx
+++ b/status/Gantt_live_11DP-C.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11020"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ettore/AI/ClaudeCode/BBI/IB/IB_Project/Submission/2026.10.20_corrections/repo/status/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ettore/AI/ClaudeCode/BBI/IB/IB_Project/Final/status_update/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBF45DA8-E833-BC4C-A433-DA12B450F61E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A98B01A5-7A4B-614E-B965-F853DA7D8B4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="17980" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -252,7 +252,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="724" uniqueCount="424">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="728" uniqueCount="430">
   <si>
     <t>Project Status · Group 11DP-C · Pyruvate Kinase Deficiency</t>
   </si>
@@ -395,13 +395,13 @@
     <t>In progress</t>
   </si>
   <si>
-    <t>Meeting of 16 Oct held; next meeting 23 Oct.</t>
+    <t>Meeting of 16 Oct held.</t>
   </si>
   <si>
     <t>1.8 Prepare the Project Status document for the 22 Oct discussion</t>
   </si>
   <si>
-    <t>This update, for the class discussion of 22 Oct.</t>
+    <t>Project Status of 20 Oct, discussed in class on 22 Oct.</t>
   </si>
   <si>
     <t>1.9 Produce the final Gantt chart with real dates (live version)</t>
@@ -416,151 +416,169 @@
     <t>2.1 Characterize the supplied sequences: translate both CDSs, compare wild type and mutant, and name the variant in HGVS nomenclature</t>
   </si>
   <si>
-    <t>Variant c.1456C&gt;T, p.Arg486Trp (missense) identified in the sequence alignment lab (lab/Lab_1_.md); translation of both CDSs to be documented.</t>
+    <t>Both CDSs translated; one difference, c.1456C&gt;T, p.(Arg486Trp).</t>
   </si>
   <si>
     <t>2.2 Identify the gene, the isoform, and the reference entries (HGNC, NCBI Gene, UniProt)</t>
   </si>
   <si>
-    <t>NCBI Gene 5313, RefSeq NM_000298.6 and NP_000289.1, and OMIM recorded in lab/Lab_1_.md; HGNC:9020 and UniProt P30613 to be added.</t>
+    <t>Reference records in analysis/sequence/raw/.</t>
   </si>
   <si>
     <t>2.3 Collect clinical and population evidence on the variant (ClinVar, gnomAD, OMIM, literature)</t>
   </si>
   <si>
+    <t>ClinVar and gnomAD evidence; Table 1.</t>
+  </si>
+  <si>
+    <t>2.4 Review the literature on PK and PKD: normal function, mechanism, inheritance, and clinical features</t>
+  </si>
+  <si>
+    <t>Literature search committed; source articles and records for references/ to be added.</t>
+  </si>
+  <si>
+    <t>2.5 Retrieve the reviewed orthologous sequences: rat, mouse, and dog (outgroup)</t>
+  </si>
+  <si>
+    <t>Rat, mouse, and dog PKLR and the vertebrate panel.</t>
+  </si>
+  <si>
+    <t>2.6 Select the experimental structures: wild-type and mutant human R-type PK; rat PK</t>
+  </si>
+  <si>
+    <t>Structure selection under way; remaining structure files to be added.</t>
+  </si>
+  <si>
+    <t>2.7 Archive the sources in references/ and maintain the reference list</t>
+  </si>
+  <si>
+    <t>Database records added to references/databases/; reference list to be completed.</t>
+  </si>
+  <si>
+    <t>2.8 Verify the sequence characterization independently: repeat the translation and the comparison of the four files</t>
+  </si>
+  <si>
+    <t>Translation, variant, and identities recomputed by independent methods: all agree.</t>
+  </si>
+  <si>
+    <t>WP3 · Sequence and structure analysis</t>
+  </si>
+  <si>
+    <t>3.1 Pairwise alignments of human PK with the rat and mouse orthologs (protein and CDS)</t>
+  </si>
+  <si>
+    <t>Human PKLR vs rat, mouse, and dog: protein identity 91.1%, 91.6%, 92.5%.</t>
+  </si>
+  <si>
+    <t>3.2 Multiple sequence alignment of human, rat, mouse, and dog PK; conservation of the substituted position and lineage of each difference</t>
+  </si>
+  <si>
+    <t>Multiple alignments; residue 486 by species; Figure 1, Table 2.</t>
+  </si>
+  <si>
+    <t>3.3 Map the substituted residue on the wild-type structure: distances to the active site, the allosteric site, and the domain and subunit interfaces</t>
+  </si>
+  <si>
+    <t>Arg486 in the C domain; distances to the FBP and active sites.</t>
+  </si>
+  <si>
+    <t>3.4 Superpose the wild-type and mutant structures (repeated in the 22 Oct lab)</t>
+  </si>
+  <si>
+    <t>Wild-type and R486W structures superposed.</t>
+  </si>
+  <si>
+    <t>3.5 Compare the human R-type and rat L-type structures around the substituted position</t>
+  </si>
+  <si>
+    <t>Human and rat structures compared; Figure 3 committed, Figure 2 to be added.</t>
+  </si>
+  <si>
+    <t>3.6 Assess pathogenicity: combine clinical, population, conservation, structural, and biochemical evidence</t>
+  </si>
+  <si>
+    <t>To be completed with the report on 25 Oct.</t>
+  </si>
+  <si>
+    <t>3.7 Explain the impact on the patient: from enzyme activity to red-cell ATP, haemolysis, and clinical severity</t>
+  </si>
+  <si>
+    <t>3.8 Team synthesis meeting: from variant to patient</t>
+  </si>
+  <si>
+    <t>3.9 Verify the alignments independently: repeat the multiple sequence alignment and check the residue at the substituted position in every species</t>
+  </si>
+  <si>
+    <t>Residue 486 checked across vertebrate PKLR orthologues.</t>
+  </si>
+  <si>
+    <t>WP4 · Report, delivery, and defence</t>
+  </si>
+  <si>
+    <t>4.1 Write the Background</t>
+  </si>
+  <si>
+    <t>Background committed.</t>
+  </si>
+  <si>
+    <t>4.2 Write the Methods</t>
+  </si>
+  <si>
+    <t>4.3 Write the Results on sequences and species comparison</t>
+  </si>
+  <si>
+    <t>4.4 Write the Results on structures; prepare the figures</t>
+  </si>
+  <si>
+    <t>4.5 Write the Discussion and Conclusions</t>
+  </si>
+  <si>
+    <t>4.6 Write the Abstract and assemble the report</t>
+  </si>
+  <si>
+    <t>4.7 Coordinate the full read-through and corrections</t>
+  </si>
+  <si>
+    <t>4.8 Check the format limits and the references</t>
+  </si>
+  <si>
+    <t>4.9 Deliver the final report on GitHub</t>
+  </si>
+  <si>
+    <t>4.10 Prepare the defence slides on the background and the impact on the patient</t>
+  </si>
+  <si>
+    <t>4.11 Prepare the defence slides on the data sources and methods</t>
+  </si>
+  <si>
+    <t>4.12 Prepare the defence slides on the discussion and conclusions</t>
+  </si>
+  <si>
+    <t>4.13 Prepare the defence slides on the sequence and species-comparison results</t>
+  </si>
+  <si>
+    <t>4.14 Prepare the defence slides on the structural results</t>
+  </si>
+  <si>
+    <t>4.15 Assemble the defence presentation: unify the format and confirm who presents each part</t>
+  </si>
+  <si>
+    <t>4.16 Coordinate the defence rehearsal, with cross-questioning between members</t>
+  </si>
+  <si>
+    <t>Legend</t>
+  </si>
+  <si>
+    <t>Canceled</t>
+  </si>
+  <si>
+    <t>Will not be done; explain why in Notes</t>
+  </si>
+  <si>
+    <t>Finished; Real Finish Date filled</t>
+  </si>
+  <si>
     <t>Incident</t>
-  </si>
-  <si>
-    <t>New dates to be set at the team meeting of 21 Oct.</t>
-  </si>
-  <si>
-    <t>2.4 Review the literature on PK and PKD: normal function, mechanism, inheritance, and clinical features</t>
-  </si>
-  <si>
-    <t>2.5 Retrieve the reviewed orthologous sequences: rat, mouse, and dog (outgroup)</t>
-  </si>
-  <si>
-    <t>Rat PKLR (NM_012624.3, NP_036756.3) recorded in lab/Lab_1_.md; mouse and dog PKLR to be retrieved.</t>
-  </si>
-  <si>
-    <t>2.6 Select the experimental structures: wild-type and mutant human R-type PK; rat PK</t>
-  </si>
-  <si>
-    <t>2.7 Archive the sources in references/ and maintain the reference list</t>
-  </si>
-  <si>
-    <t>2.8 Verify the sequence characterization independently: repeat the translation and the comparison of the four files</t>
-  </si>
-  <si>
-    <t>Follows 2.1. New dates to be set at the team meeting of 21 Oct.</t>
-  </si>
-  <si>
-    <t>WP3 · Sequence and structure analysis</t>
-  </si>
-  <si>
-    <t>3.1 Pairwise alignments of human PK with the rat and mouse orthologs (protein and CDS)</t>
-  </si>
-  <si>
-    <t>Started in the sequence alignment lab (lab/Lab_1_.md); to be completed with the PKLR sequences of rat and mouse.</t>
-  </si>
-  <si>
-    <t>3.2 Multiple sequence alignment of human, rat, mouse, and dog PK; conservation of the substituted position and lineage of each difference</t>
-  </si>
-  <si>
-    <t>Follows 2.5. New dates to be set at the team meeting of 21 Oct.</t>
-  </si>
-  <si>
-    <t>3.3 Map the substituted residue on the wild-type structure: distances to the active site, the allosteric site, and the domain and subunit interfaces</t>
-  </si>
-  <si>
-    <t>Follows 2.6. New dates to be set at the team meeting of 21 Oct.</t>
-  </si>
-  <si>
-    <t>3.4 Superpose the wild-type and mutant structures (repeated in the 22 Oct lab)</t>
-  </si>
-  <si>
-    <t>Scheduled for the structure superposition lab of 22 Oct.</t>
-  </si>
-  <si>
-    <t>3.5 Compare the human R-type and rat L-type structures around the substituted position</t>
-  </si>
-  <si>
-    <t>3.6 Assess pathogenicity: combine clinical, population, conservation, structural, and biochemical evidence</t>
-  </si>
-  <si>
-    <t>Follows 2.3 and 3.2. New dates to be set at the team meeting of 21 Oct.</t>
-  </si>
-  <si>
-    <t>3.7 Explain the impact on the patient: from enzyme activity to red-cell ATP, haemolysis, and clinical severity</t>
-  </si>
-  <si>
-    <t>3.8 Team synthesis meeting: from variant to patient</t>
-  </si>
-  <si>
-    <t>3.9 Verify the alignments independently: repeat the multiple sequence alignment and check the residue at the substituted position in every species</t>
-  </si>
-  <si>
-    <t>WP4 · Report, delivery, and defence</t>
-  </si>
-  <si>
-    <t>4.1 Write the Background</t>
-  </si>
-  <si>
-    <t>4.2 Write the Methods</t>
-  </si>
-  <si>
-    <t>4.3 Write the Results on sequences and species comparison</t>
-  </si>
-  <si>
-    <t>4.4 Write the Results on structures; prepare the figures</t>
-  </si>
-  <si>
-    <t>4.5 Write the Discussion and Conclusions</t>
-  </si>
-  <si>
-    <t>4.6 Write the Abstract and assemble the report</t>
-  </si>
-  <si>
-    <t>4.7 Coordinate the full read-through and corrections</t>
-  </si>
-  <si>
-    <t>4.8 Check the format limits and the references</t>
-  </si>
-  <si>
-    <t>4.9 Deliver the final report on GitHub</t>
-  </si>
-  <si>
-    <t>4.10 Prepare the defence slides on the background and the impact on the patient</t>
-  </si>
-  <si>
-    <t>4.11 Prepare the defence slides on the data sources and methods</t>
-  </si>
-  <si>
-    <t>4.12 Prepare the defence slides on the discussion and conclusions</t>
-  </si>
-  <si>
-    <t>4.13 Prepare the defence slides on the sequence and species-comparison results</t>
-  </si>
-  <si>
-    <t>4.14 Prepare the defence slides on the structural results</t>
-  </si>
-  <si>
-    <t>4.15 Assemble the defence presentation: unify the format and confirm who presents each part</t>
-  </si>
-  <si>
-    <t>4.16 Coordinate the defence rehearsal, with cross-questioning between members</t>
-  </si>
-  <si>
-    <t>Legend</t>
-  </si>
-  <si>
-    <t>Canceled</t>
-  </si>
-  <si>
-    <t>Will not be done; explain why in Notes</t>
-  </si>
-  <si>
-    <t>Finished; Real Finish Date filled</t>
   </si>
   <si>
     <t>A problem occurred; describe it and the workaround in Notes</t>
@@ -3063,12 +3081,12 @@
   <sheetData>
     <row r="1" spans="1:1" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
@@ -3076,37 +3094,37 @@
     </row>
     <row r="4" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
     </row>
     <row r="6" spans="1:1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
     </row>
     <row r="8" spans="1:1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
     </row>
     <row r="10" spans="1:1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.2">
@@ -3114,22 +3132,22 @@
     </row>
     <row r="12" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A13" s="5" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A14" s="5" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
     </row>
     <row r="15" spans="1:1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="5" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.2">
@@ -3137,17 +3155,17 @@
     </row>
     <row r="17" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
     </row>
     <row r="18" spans="1:1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="5" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A19" s="5" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.2">
@@ -3155,22 +3173,22 @@
     </row>
     <row r="21" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="4" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
     </row>
     <row r="22" spans="1:1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="5" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
     </row>
     <row r="23" spans="1:1" ht="56" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="5" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A26" s="6" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
     </row>
   </sheetData>
@@ -3203,7 +3221,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="9">
-        <v>46315</v>
+        <v>46319</v>
       </c>
       <c r="C2" s="10" t="s">
         <v>2</v>
@@ -3723,9 +3741,11 @@
       <c r="E23" s="17">
         <v>46315</v>
       </c>
-      <c r="F23" s="17"/>
+      <c r="F23" s="17">
+        <v>46315</v>
+      </c>
       <c r="G23" s="18" t="s">
-        <v>46</v>
+        <v>14</v>
       </c>
       <c r="H23" s="19" t="s">
         <v>49</v>
@@ -3740,11 +3760,11 @@
       </c>
       <c r="C24" s="16">
         <f>Tasks!H24</f>
-        <v>46322</v>
+        <v>46321</v>
       </c>
       <c r="D24" s="16">
         <f>Tasks!I24</f>
-        <v>46322</v>
+        <v>46321</v>
       </c>
       <c r="E24" s="17"/>
       <c r="F24" s="17"/>
@@ -3774,18 +3794,20 @@
       </c>
       <c r="C26" s="16">
         <f>Tasks!H26</f>
-        <v>46308</v>
+        <v>46318</v>
       </c>
       <c r="D26" s="16">
         <f>Tasks!I26</f>
-        <v>46308</v>
+        <v>46318</v>
       </c>
       <c r="E26" s="17">
-        <v>46314</v>
-      </c>
-      <c r="F26" s="17"/>
+        <v>46318</v>
+      </c>
+      <c r="F26" s="17">
+        <v>46319</v>
+      </c>
       <c r="G26" s="18" t="s">
-        <v>46</v>
+        <v>14</v>
       </c>
       <c r="H26" s="19" t="s">
         <v>54</v>
@@ -3800,18 +3822,20 @@
       </c>
       <c r="C27" s="16">
         <f>Tasks!H27</f>
-        <v>46308</v>
+        <v>46318</v>
       </c>
       <c r="D27" s="16">
         <f>Tasks!I27</f>
-        <v>46308</v>
+        <v>46318</v>
       </c>
       <c r="E27" s="17">
-        <v>46314</v>
-      </c>
-      <c r="F27" s="17"/>
+        <v>46319</v>
+      </c>
+      <c r="F27" s="17">
+        <v>46319</v>
+      </c>
       <c r="G27" s="18" t="s">
-        <v>46</v>
+        <v>14</v>
       </c>
       <c r="H27" s="19" t="s">
         <v>56</v>
@@ -3826,43 +3850,49 @@
       </c>
       <c r="C28" s="16">
         <f>Tasks!H28</f>
-        <v>46310</v>
+        <v>46318</v>
       </c>
       <c r="D28" s="16">
         <f>Tasks!I28</f>
-        <v>46311</v>
-      </c>
-      <c r="E28" s="17"/>
-      <c r="F28" s="17"/>
+        <v>46318</v>
+      </c>
+      <c r="E28" s="17">
+        <v>46319</v>
+      </c>
+      <c r="F28" s="17">
+        <v>46319</v>
+      </c>
       <c r="G28" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="H28" s="19" t="s">
         <v>58</v>
-      </c>
-      <c r="H28" s="19" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="29" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="14" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B29" s="22" t="s">
         <v>23</v>
       </c>
       <c r="C29" s="16">
         <f>Tasks!H29</f>
-        <v>46308</v>
+        <v>46318</v>
       </c>
       <c r="D29" s="16">
         <f>Tasks!I29</f>
-        <v>46310</v>
-      </c>
-      <c r="E29" s="17"/>
+        <v>46319</v>
+      </c>
+      <c r="E29" s="17">
+        <v>46318</v>
+      </c>
       <c r="F29" s="17"/>
       <c r="G29" s="18" t="s">
-        <v>58</v>
+        <v>46</v>
       </c>
       <c r="H29" s="19" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.2">
@@ -3874,18 +3904,20 @@
       </c>
       <c r="C30" s="16">
         <f>Tasks!H30</f>
-        <v>46309</v>
+        <v>46318</v>
       </c>
       <c r="D30" s="16">
         <f>Tasks!I30</f>
-        <v>46309</v>
+        <v>46318</v>
       </c>
       <c r="E30" s="17">
-        <v>46314</v>
-      </c>
-      <c r="F30" s="17"/>
+        <v>46319</v>
+      </c>
+      <c r="F30" s="17">
+        <v>46319</v>
+      </c>
       <c r="G30" s="18" t="s">
-        <v>46</v>
+        <v>14</v>
       </c>
       <c r="H30" s="19" t="s">
         <v>62</v>
@@ -3900,72 +3932,80 @@
       </c>
       <c r="C31" s="16">
         <f>Tasks!H31</f>
-        <v>46308</v>
+        <v>46318</v>
       </c>
       <c r="D31" s="16">
         <f>Tasks!I31</f>
-        <v>46308</v>
-      </c>
-      <c r="E31" s="17"/>
+        <v>46318</v>
+      </c>
+      <c r="E31" s="17">
+        <v>46319</v>
+      </c>
       <c r="F31" s="17"/>
       <c r="G31" s="18" t="s">
-        <v>58</v>
+        <v>46</v>
       </c>
       <c r="H31" s="19" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
     </row>
     <row r="32" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="14" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B32" s="15" t="s">
         <v>13</v>
       </c>
       <c r="C32" s="16">
         <f>Tasks!H32</f>
-        <v>46314</v>
+        <v>46319</v>
       </c>
       <c r="D32" s="16">
         <f>Tasks!I32</f>
-        <v>46314</v>
-      </c>
-      <c r="E32" s="17"/>
+        <v>46320</v>
+      </c>
+      <c r="E32" s="17">
+        <v>46319</v>
+      </c>
       <c r="F32" s="17"/>
       <c r="G32" s="18" t="s">
-        <v>58</v>
+        <v>46</v>
       </c>
       <c r="H32" s="19" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
     </row>
     <row r="33" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="14" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B33" s="20" t="s">
         <v>17</v>
       </c>
       <c r="C33" s="16">
         <f>Tasks!H33</f>
-        <v>46309</v>
+        <v>46318</v>
       </c>
       <c r="D33" s="16">
         <f>Tasks!I33</f>
-        <v>46309</v>
-      </c>
-      <c r="E33" s="17"/>
-      <c r="F33" s="17"/>
+        <v>46318</v>
+      </c>
+      <c r="E33" s="17">
+        <v>46319</v>
+      </c>
+      <c r="F33" s="17">
+        <v>46319</v>
+      </c>
       <c r="G33" s="18" t="s">
-        <v>58</v>
+        <v>14</v>
       </c>
       <c r="H33" s="19" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A34" s="29" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B34" s="30"/>
       <c r="C34" s="30"/>
@@ -3977,184 +4017,204 @@
     </row>
     <row r="35" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="14" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B35" s="25" t="s">
         <v>36</v>
       </c>
       <c r="C35" s="16">
         <f>Tasks!H35</f>
-        <v>46310</v>
+        <v>46318</v>
       </c>
       <c r="D35" s="16">
         <f>Tasks!I35</f>
-        <v>46310</v>
+        <v>46318</v>
       </c>
       <c r="E35" s="17">
-        <v>46314</v>
-      </c>
-      <c r="F35" s="17"/>
+        <v>46318</v>
+      </c>
+      <c r="F35" s="17">
+        <v>46319</v>
+      </c>
       <c r="G35" s="18" t="s">
-        <v>46</v>
+        <v>14</v>
       </c>
       <c r="H35" s="19" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="36" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="14" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B36" s="25" t="s">
         <v>36</v>
       </c>
       <c r="C36" s="16">
         <f>Tasks!H36</f>
-        <v>46311</v>
+        <v>46319</v>
       </c>
       <c r="D36" s="16">
         <f>Tasks!I36</f>
-        <v>46314</v>
-      </c>
-      <c r="E36" s="17"/>
-      <c r="F36" s="17"/>
+        <v>46319</v>
+      </c>
+      <c r="E36" s="17">
+        <v>46319</v>
+      </c>
+      <c r="F36" s="17">
+        <v>46319</v>
+      </c>
       <c r="G36" s="18" t="s">
-        <v>58</v>
+        <v>14</v>
       </c>
       <c r="H36" s="19" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="37" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="14" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B37" s="26" t="s">
         <v>39</v>
       </c>
       <c r="C37" s="16">
         <f>Tasks!H37</f>
-        <v>46309</v>
+        <v>46318</v>
       </c>
       <c r="D37" s="16">
         <f>Tasks!I37</f>
-        <v>46310</v>
-      </c>
-      <c r="E37" s="17"/>
-      <c r="F37" s="17"/>
+        <v>46318</v>
+      </c>
+      <c r="E37" s="17">
+        <v>46319</v>
+      </c>
+      <c r="F37" s="17">
+        <v>46319</v>
+      </c>
       <c r="G37" s="18" t="s">
-        <v>58</v>
+        <v>14</v>
       </c>
       <c r="H37" s="19" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="38" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="14" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B38" s="26" t="s">
         <v>39</v>
       </c>
       <c r="C38" s="16">
         <f>Tasks!H38</f>
-        <v>46311</v>
+        <v>46319</v>
       </c>
       <c r="D38" s="16">
         <f>Tasks!I38</f>
-        <v>46314</v>
-      </c>
-      <c r="E38" s="17"/>
-      <c r="F38" s="17"/>
+        <v>46319</v>
+      </c>
+      <c r="E38" s="17">
+        <v>46319</v>
+      </c>
+      <c r="F38" s="17">
+        <v>46319</v>
+      </c>
       <c r="G38" s="18" t="s">
-        <v>58</v>
+        <v>14</v>
       </c>
       <c r="H38" s="19" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="14" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B39" s="26" t="s">
         <v>39</v>
       </c>
       <c r="C39" s="16">
         <f>Tasks!H39</f>
-        <v>46315</v>
+        <v>46319</v>
       </c>
       <c r="D39" s="16">
         <f>Tasks!I39</f>
-        <v>46315</v>
-      </c>
-      <c r="E39" s="17"/>
+        <v>46319</v>
+      </c>
+      <c r="E39" s="17">
+        <v>46319</v>
+      </c>
       <c r="F39" s="17"/>
       <c r="G39" s="18" t="s">
-        <v>51</v>
-      </c>
-      <c r="H39" s="19"/>
+        <v>46</v>
+      </c>
+      <c r="H39" s="19" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="40" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="14" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="B40" s="22" t="s">
         <v>23</v>
       </c>
       <c r="C40" s="16">
         <f>Tasks!H40</f>
-        <v>46314</v>
+        <v>46319</v>
       </c>
       <c r="D40" s="16">
         <f>Tasks!I40</f>
-        <v>46314</v>
+        <v>46319</v>
       </c>
       <c r="E40" s="17"/>
       <c r="F40" s="17"/>
       <c r="G40" s="18" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="H40" s="19" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
     </row>
     <row r="41" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="14" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="B41" s="22" t="s">
         <v>23</v>
       </c>
       <c r="C41" s="16">
         <f>Tasks!H41</f>
-        <v>46315</v>
+        <v>46319</v>
       </c>
       <c r="D41" s="16">
         <f>Tasks!I41</f>
-        <v>46315</v>
+        <v>46319</v>
       </c>
       <c r="E41" s="17"/>
       <c r="F41" s="17"/>
       <c r="G41" s="18" t="s">
         <v>51</v>
       </c>
-      <c r="H41" s="19"/>
+      <c r="H41" s="19" t="s">
+        <v>81</v>
+      </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A42" s="14" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B42" s="20" t="s">
         <v>17</v>
       </c>
       <c r="C42" s="16">
         <f>Tasks!H42</f>
-        <v>46316</v>
+        <v>46320</v>
       </c>
       <c r="D42" s="16">
         <f>Tasks!I42</f>
-        <v>46316</v>
+        <v>46320</v>
       </c>
       <c r="E42" s="17"/>
       <c r="F42" s="17"/>
@@ -4165,29 +4225,35 @@
     </row>
     <row r="43" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="14" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B43" s="15" t="s">
         <v>13</v>
       </c>
       <c r="C43" s="16">
         <f>Tasks!H43</f>
-        <v>46315</v>
+        <v>46319</v>
       </c>
       <c r="D43" s="16">
         <f>Tasks!I43</f>
-        <v>46315</v>
-      </c>
-      <c r="E43" s="17"/>
-      <c r="F43" s="17"/>
+        <v>46319</v>
+      </c>
+      <c r="E43" s="17">
+        <v>46319</v>
+      </c>
+      <c r="F43" s="17">
+        <v>46319</v>
+      </c>
       <c r="G43" s="18" t="s">
-        <v>51</v>
-      </c>
-      <c r="H43" s="19"/>
+        <v>14</v>
+      </c>
+      <c r="H43" s="19" t="s">
+        <v>85</v>
+      </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A44" s="31" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="B44" s="32"/>
       <c r="C44" s="32"/>
@@ -4199,40 +4265,44 @@
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A45" s="14" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="B45" s="22" t="s">
         <v>23</v>
       </c>
       <c r="C45" s="16">
         <f>Tasks!H45</f>
-        <v>46316</v>
+        <v>46319</v>
       </c>
       <c r="D45" s="16">
         <f>Tasks!I45</f>
-        <v>46317</v>
-      </c>
-      <c r="E45" s="17"/>
+        <v>46319</v>
+      </c>
+      <c r="E45" s="17">
+        <v>46319</v>
+      </c>
       <c r="F45" s="17"/>
       <c r="G45" s="18" t="s">
-        <v>51</v>
-      </c>
-      <c r="H45" s="19"/>
+        <v>46</v>
+      </c>
+      <c r="H45" s="19" t="s">
+        <v>88</v>
+      </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A46" s="14" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="B46" s="15" t="s">
         <v>13</v>
       </c>
       <c r="C46" s="16">
         <f>Tasks!H46</f>
-        <v>46316</v>
+        <v>46320</v>
       </c>
       <c r="D46" s="16">
         <f>Tasks!I46</f>
-        <v>46317</v>
+        <v>46320</v>
       </c>
       <c r="E46" s="17"/>
       <c r="F46" s="17"/>
@@ -4243,18 +4313,18 @@
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A47" s="14" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="B47" s="25" t="s">
         <v>36</v>
       </c>
       <c r="C47" s="16">
         <f>Tasks!H47</f>
-        <v>46315</v>
+        <v>46320</v>
       </c>
       <c r="D47" s="16">
         <f>Tasks!I47</f>
-        <v>46316</v>
+        <v>46320</v>
       </c>
       <c r="E47" s="17"/>
       <c r="F47" s="17"/>
@@ -4265,18 +4335,18 @@
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A48" s="14" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="B48" s="26" t="s">
         <v>39</v>
       </c>
       <c r="C48" s="16">
         <f>Tasks!H48</f>
-        <v>46316</v>
+        <v>46320</v>
       </c>
       <c r="D48" s="16">
         <f>Tasks!I48</f>
-        <v>46317</v>
+        <v>46320</v>
       </c>
       <c r="E48" s="17"/>
       <c r="F48" s="17"/>
@@ -4287,18 +4357,18 @@
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A49" s="14" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="B49" s="20" t="s">
         <v>17</v>
       </c>
       <c r="C49" s="16">
         <f>Tasks!H49</f>
-        <v>46317</v>
+        <v>46320</v>
       </c>
       <c r="D49" s="16">
         <f>Tasks!I49</f>
-        <v>46318</v>
+        <v>46320</v>
       </c>
       <c r="E49" s="17"/>
       <c r="F49" s="17"/>
@@ -4309,7 +4379,7 @@
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A50" s="14" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="B50" s="22" t="s">
         <v>23</v>
@@ -4331,18 +4401,18 @@
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A51" s="14" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="B51" s="25" t="s">
         <v>36</v>
       </c>
       <c r="C51" s="16">
         <f>Tasks!H51</f>
-        <v>46322</v>
+        <v>46321</v>
       </c>
       <c r="D51" s="16">
         <f>Tasks!I51</f>
-        <v>46322</v>
+        <v>46321</v>
       </c>
       <c r="E51" s="17"/>
       <c r="F51" s="17"/>
@@ -4353,18 +4423,18 @@
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A52" s="14" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="B52" s="15" t="s">
         <v>13</v>
       </c>
       <c r="C52" s="16">
         <f>Tasks!H52</f>
-        <v>46322</v>
+        <v>46321</v>
       </c>
       <c r="D52" s="16">
         <f>Tasks!I52</f>
-        <v>46322</v>
+        <v>46321</v>
       </c>
       <c r="E52" s="17"/>
       <c r="F52" s="17"/>
@@ -4375,18 +4445,18 @@
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A53" s="14" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="B53" s="22" t="s">
         <v>23</v>
       </c>
       <c r="C53" s="16">
         <f>Tasks!H53</f>
-        <v>46323</v>
+        <v>46321</v>
       </c>
       <c r="D53" s="16">
         <f>Tasks!I53</f>
-        <v>46323</v>
+        <v>46321</v>
       </c>
       <c r="E53" s="17"/>
       <c r="F53" s="17"/>
@@ -4397,18 +4467,18 @@
     </row>
     <row r="54" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="14" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="B54" s="22" t="s">
         <v>23</v>
       </c>
       <c r="C54" s="16">
         <f>Tasks!H54</f>
-        <v>46324</v>
+        <v>46322</v>
       </c>
       <c r="D54" s="16">
         <f>Tasks!I54</f>
-        <v>46324</v>
+        <v>46322</v>
       </c>
       <c r="E54" s="17"/>
       <c r="F54" s="17"/>
@@ -4419,18 +4489,18 @@
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A55" s="14" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="B55" s="15" t="s">
         <v>13</v>
       </c>
       <c r="C55" s="16">
         <f>Tasks!H55</f>
-        <v>46324</v>
+        <v>46322</v>
       </c>
       <c r="D55" s="16">
         <f>Tasks!I55</f>
-        <v>46324</v>
+        <v>46322</v>
       </c>
       <c r="E55" s="17"/>
       <c r="F55" s="17"/>
@@ -4441,18 +4511,18 @@
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A56" s="14" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="B56" s="20" t="s">
         <v>17</v>
       </c>
       <c r="C56" s="16">
         <f>Tasks!H56</f>
-        <v>46324</v>
+        <v>46322</v>
       </c>
       <c r="D56" s="16">
         <f>Tasks!I56</f>
-        <v>46324</v>
+        <v>46322</v>
       </c>
       <c r="E56" s="17"/>
       <c r="F56" s="17"/>
@@ -4463,18 +4533,18 @@
     </row>
     <row r="57" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="14" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="B57" s="25" t="s">
         <v>36</v>
       </c>
       <c r="C57" s="16">
         <f>Tasks!H57</f>
-        <v>46324</v>
+        <v>46322</v>
       </c>
       <c r="D57" s="16">
         <f>Tasks!I57</f>
-        <v>46324</v>
+        <v>46322</v>
       </c>
       <c r="E57" s="17"/>
       <c r="F57" s="17"/>
@@ -4485,18 +4555,18 @@
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A58" s="14" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="B58" s="26" t="s">
         <v>39</v>
       </c>
       <c r="C58" s="16">
         <f>Tasks!H58</f>
-        <v>46324</v>
+        <v>46322</v>
       </c>
       <c r="D58" s="16">
         <f>Tasks!I58</f>
-        <v>46324</v>
+        <v>46322</v>
       </c>
       <c r="E58" s="17"/>
       <c r="F58" s="17"/>
@@ -4507,7 +4577,7 @@
     </row>
     <row r="59" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="14" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="B59" s="15" t="s">
         <v>13</v>
@@ -4529,7 +4599,7 @@
     </row>
     <row r="60" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="14" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="B60" s="25" t="s">
         <v>36</v>
@@ -4551,15 +4621,15 @@
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A62" s="33" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A63" s="34" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="B63" s="35" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.2">
@@ -4567,15 +4637,15 @@
         <v>14</v>
       </c>
       <c r="B64" s="35" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A65" s="37" t="s">
-        <v>58</v>
+        <v>108</v>
       </c>
       <c r="B65" s="35" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.2">
@@ -4583,15 +4653,15 @@
         <v>46</v>
       </c>
       <c r="B66" s="35" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A67" s="39" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="B67" s="35" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.2">
@@ -4599,12 +4669,12 @@
         <v>51</v>
       </c>
       <c r="B68" s="35" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A70" s="10" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
     </row>
   </sheetData>
@@ -4675,12 +4745,12 @@
   <sheetData>
     <row r="1" spans="1:50" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="41" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A2" s="10" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
     </row>
     <row r="3" spans="1:50" x14ac:dyDescent="0.2">
@@ -4739,43 +4809,43 @@
     </row>
     <row r="4" spans="1:50" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="11" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="C4" s="11" t="s">
         <v>3</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="F4" s="11" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="G4" s="11" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="H4" s="11" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="I4" s="11" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="J4" s="11" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="K4" s="11" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="L4" s="11" t="s">
         <v>9</v>
       </c>
       <c r="M4" s="11" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="N4" s="42">
         <v>46282</v>
@@ -4886,15 +4956,15 @@
         <v>46331</v>
       </c>
       <c r="AX4" s="11" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
     </row>
     <row r="5" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A5" s="12" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="C5" s="13" t="s">
         <v>11</v>
@@ -4957,13 +5027,13 @@
     </row>
     <row r="6" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A6" s="45" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="B6" s="45" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="C6" s="45" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="D6" s="46" t="s">
         <v>13</v>
@@ -5143,18 +5213,18 @@
         <v/>
       </c>
       <c r="AX6" s="49" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
     </row>
     <row r="7" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A7" s="45" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="B7" s="45" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="C7" s="45" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="D7" s="50" t="s">
         <v>17</v>
@@ -5334,18 +5404,18 @@
         <v/>
       </c>
       <c r="AX7" s="49" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
     </row>
     <row r="8" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A8" s="45" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="B8" s="45" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="C8" s="45" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="D8" s="51" t="s">
         <v>19</v>
@@ -5525,18 +5595,18 @@
         <v/>
       </c>
       <c r="AX8" s="49" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
     </row>
     <row r="9" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A9" s="45" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="B9" s="45" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="C9" s="45" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="D9" s="51" t="s">
         <v>19</v>
@@ -5716,18 +5786,18 @@
         <v/>
       </c>
       <c r="AX9" s="49" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
     </row>
     <row r="10" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A10" s="45" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="B10" s="45" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="C10" s="45" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="D10" s="52" t="s">
         <v>23</v>
@@ -5907,18 +5977,18 @@
         <v/>
       </c>
       <c r="AX10" s="49" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
     </row>
     <row r="11" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A11" s="45" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="B11" s="45" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="C11" s="45" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="D11" s="51" t="s">
         <v>19</v>
@@ -6098,18 +6168,18 @@
         <v/>
       </c>
       <c r="AX11" s="49" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
     </row>
     <row r="12" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A12" s="45" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="B12" s="45" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="C12" s="45" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="D12" s="51" t="s">
         <v>19</v>
@@ -6289,18 +6359,18 @@
         <v/>
       </c>
       <c r="AX12" s="49" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
     </row>
     <row r="13" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A13" s="45" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="B13" s="45" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="C13" s="45" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="D13" s="50" t="s">
         <v>17</v>
@@ -6480,18 +6550,18 @@
         <v/>
       </c>
       <c r="AX13" s="49" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
     </row>
     <row r="14" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A14" s="45" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="B14" s="45" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="C14" s="45" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="D14" s="51" t="s">
         <v>19</v>
@@ -6671,15 +6741,15 @@
         <v/>
       </c>
       <c r="AX14" s="49" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
     </row>
     <row r="15" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A15" s="23" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="B15" s="24" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="C15" s="24" t="s">
         <v>30</v>
@@ -6687,7 +6757,7 @@
       <c r="D15" s="24"/>
       <c r="E15" s="24">
         <f>NETWORKDAYS(H15,I15,Holidays!$A$2:$A$40)</f>
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F15" s="24"/>
       <c r="G15" s="24"/>
@@ -6697,7 +6767,7 @@
       </c>
       <c r="I15" s="53">
         <f>MAX(I16:I24)</f>
-        <v>46322</v>
+        <v>46321</v>
       </c>
       <c r="J15" s="24"/>
       <c r="K15" s="24"/>
@@ -6742,13 +6812,13 @@
     </row>
     <row r="16" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A16" s="45" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
       <c r="B16" s="45" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="C16" s="45" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="D16" s="50" t="s">
         <v>17</v>
@@ -6928,18 +6998,18 @@
         <v/>
       </c>
       <c r="AX16" s="49" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
     </row>
     <row r="17" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A17" s="45" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="B17" s="45" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="C17" s="45" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="D17" s="52" t="s">
         <v>23</v>
@@ -6951,7 +7021,7 @@
         <v>1</v>
       </c>
       <c r="G17" s="45" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
       <c r="H17" s="47">
         <v>46304</v>
@@ -7121,18 +7191,18 @@
         <v/>
       </c>
       <c r="AX17" s="49" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
     </row>
     <row r="18" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A18" s="45" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="B18" s="45" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="C18" s="45" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
       <c r="D18" s="54" t="s">
         <v>36</v>
@@ -7144,7 +7214,7 @@
         <v>1</v>
       </c>
       <c r="G18" s="45" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
       <c r="H18" s="47">
         <v>46304</v>
@@ -7314,18 +7384,18 @@
         <v/>
       </c>
       <c r="AX18" s="49" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
     </row>
     <row r="19" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A19" s="45" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="B19" s="45" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="C19" s="45" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="D19" s="55" t="s">
         <v>39</v>
@@ -7337,7 +7407,7 @@
         <v>1</v>
       </c>
       <c r="G19" s="45" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
       <c r="H19" s="47">
         <v>46304</v>
@@ -7507,18 +7577,18 @@
         <v/>
       </c>
       <c r="AX19" s="49" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
     </row>
     <row r="20" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A20" s="45" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="B20" s="45" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="C20" s="45" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="D20" s="46" t="s">
         <v>13</v>
@@ -7530,7 +7600,7 @@
         <v>1</v>
       </c>
       <c r="G20" s="45" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
       <c r="H20" s="47">
         <v>46304</v>
@@ -7700,18 +7770,18 @@
         <v/>
       </c>
       <c r="AX20" s="49" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
     </row>
     <row r="21" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A21" s="45" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="B21" s="45" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="C21" s="45" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
       <c r="D21" s="50" t="s">
         <v>17</v>
@@ -7723,7 +7793,7 @@
         <v>1</v>
       </c>
       <c r="G21" s="45" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="H21" s="47">
         <v>46308</v>
@@ -7893,18 +7963,18 @@
         <v/>
       </c>
       <c r="AX21" s="49" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
     </row>
     <row r="22" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A22" s="45" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="B22" s="45" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="C22" s="45" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="D22" s="50" t="s">
         <v>17</v>
@@ -7916,7 +7986,7 @@
         <v>2</v>
       </c>
       <c r="G22" s="45" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="H22" s="47">
         <v>46311</v>
@@ -8039,15 +8109,15 @@
       </c>
       <c r="AL22" s="48" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v/>
+        <v>●</v>
       </c>
       <c r="AM22" s="48" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v/>
+        <v>●</v>
       </c>
       <c r="AN22" s="48" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v/>
+        <v>●</v>
       </c>
       <c r="AO22" s="48" t="str">
         <f t="shared" ca="1" si="6"/>
@@ -8086,18 +8156,18 @@
         <v/>
       </c>
       <c r="AX22" s="49" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
     </row>
     <row r="23" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A23" s="45" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="B23" s="45" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="C23" s="45" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="D23" s="50" t="s">
         <v>17</v>
@@ -8109,7 +8179,7 @@
         <v>1</v>
       </c>
       <c r="G23" s="45" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="H23" s="47">
         <v>46315</v>
@@ -8122,17 +8192,17 @@
         <f>IF('Project Status'!E23="","",'Project Status'!E23)</f>
         <v>46315</v>
       </c>
-      <c r="K23" s="47" t="str">
+      <c r="K23" s="47">
         <f>IF('Project Status'!F23="","",'Project Status'!F23)</f>
-        <v/>
+        <v>46315</v>
       </c>
       <c r="L23" s="45" t="str">
         <f>IF('Project Status'!G23="","",'Project Status'!G23)</f>
-        <v>In progress</v>
-      </c>
-      <c r="M23" s="45" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="M23" s="45">
         <f>IF(OR(K23="",I23=""),"",IF(K23&gt;=I23,NETWORKDAYS(I23,K23,Holidays!$A$2:$A$40)-1,-(NETWORKDAYS(K23,I23,Holidays!$A$2:$A$40)-1)))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N23" s="48" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -8279,18 +8349,18 @@
         <v/>
       </c>
       <c r="AX23" s="49" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
     </row>
     <row r="24" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A24" s="45" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
       <c r="B24" s="45" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="C24" s="45" t="s">
-        <v>195</v>
+        <v>201</v>
       </c>
       <c r="D24" s="50" t="s">
         <v>17</v>
@@ -8302,14 +8372,13 @@
         <v>1</v>
       </c>
       <c r="G24" s="45" t="s">
-        <v>196</v>
+        <v>202</v>
       </c>
       <c r="H24" s="47">
-        <v>46322</v>
+        <v>46321</v>
       </c>
       <c r="I24" s="47">
-        <f>WORKDAY(H24,E24-1,Holidays!$A$2:$A$40)</f>
-        <v>46322</v>
+        <v>46321</v>
       </c>
       <c r="J24" s="47" t="str">
         <f>IF('Project Status'!E24="","",'Project Status'!E24)</f>
@@ -8472,15 +8541,15 @@
         <v/>
       </c>
       <c r="AX24" s="49" t="s">
-        <v>197</v>
+        <v>203</v>
       </c>
     </row>
     <row r="25" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A25" s="27" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="B25" s="28" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="C25" s="28" t="s">
         <v>52</v>
@@ -8488,17 +8557,17 @@
       <c r="D25" s="28"/>
       <c r="E25" s="28">
         <f>NETWORKDAYS(H25,I25,Holidays!$A$2:$A$40)</f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F25" s="28"/>
       <c r="G25" s="28"/>
       <c r="H25" s="56">
         <f>MIN(H26:H33)</f>
-        <v>46308</v>
+        <v>46318</v>
       </c>
       <c r="I25" s="56">
         <f>MAX(I26:I33)</f>
-        <v>46314</v>
+        <v>46320</v>
       </c>
       <c r="J25" s="28"/>
       <c r="K25" s="28"/>
@@ -8543,13 +8612,13 @@
     </row>
     <row r="26" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A26" s="45" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="B26" s="45" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="C26" s="45" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="D26" s="54" t="s">
         <v>36</v>
@@ -8561,30 +8630,29 @@
         <v>1</v>
       </c>
       <c r="G26" s="45" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="H26" s="47">
-        <v>46308</v>
+        <v>46318</v>
       </c>
       <c r="I26" s="47">
-        <f>WORKDAY(H26,E26-1,Holidays!$A$2:$A$40)</f>
-        <v>46308</v>
+        <v>46318</v>
       </c>
       <c r="J26" s="47">
         <f>IF('Project Status'!E26="","",'Project Status'!E26)</f>
-        <v>46314</v>
-      </c>
-      <c r="K26" s="47" t="str">
+        <v>46318</v>
+      </c>
+      <c r="K26" s="47">
         <f>IF('Project Status'!F26="","",'Project Status'!F26)</f>
-        <v/>
+        <v>46319</v>
       </c>
       <c r="L26" s="45" t="str">
         <f>IF('Project Status'!G26="","",'Project Status'!G26)</f>
-        <v>In progress</v>
-      </c>
-      <c r="M26" s="45" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="M26" s="45">
         <f>IF(OR(K26="",I26=""),"",IF(K26&gt;=I26,NETWORKDAYS(I26,K26,Holidays!$A$2:$A$40)-1,-(NETWORKDAYS(K26,I26,Holidays!$A$2:$A$40)-1)))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N26" s="48" t="str">
         <f t="shared" ref="N26:W33" ca="1" si="8">IF(AND($J26&lt;&gt;"",N$4&gt;=$J26,N$4&lt;=IF($K26="",TODAY(),$K26),N$65=0),"●","")</f>
@@ -8676,11 +8744,11 @@
       </c>
       <c r="AJ26" s="48" t="str">
         <f t="shared" ca="1" si="10"/>
-        <v>●</v>
+        <v/>
       </c>
       <c r="AK26" s="48" t="str">
         <f t="shared" ca="1" si="10"/>
-        <v>●</v>
+        <v/>
       </c>
       <c r="AL26" s="48" t="str">
         <f t="shared" ca="1" si="10"/>
@@ -8692,7 +8760,7 @@
       </c>
       <c r="AN26" s="48" t="str">
         <f t="shared" ca="1" si="10"/>
-        <v/>
+        <v>●</v>
       </c>
       <c r="AO26" s="48" t="str">
         <f t="shared" ca="1" si="10"/>
@@ -8731,18 +8799,18 @@
         <v/>
       </c>
       <c r="AX26" s="49" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
     </row>
     <row r="27" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A27" s="45" t="s">
-        <v>202</v>
+        <v>208</v>
       </c>
       <c r="B27" s="45" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="C27" s="45" t="s">
-        <v>203</v>
+        <v>209</v>
       </c>
       <c r="D27" s="46" t="s">
         <v>13</v>
@@ -8754,30 +8822,29 @@
         <v>1</v>
       </c>
       <c r="G27" s="45" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="H27" s="47">
-        <v>46308</v>
+        <v>46318</v>
       </c>
       <c r="I27" s="47">
-        <f>WORKDAY(H27,E27-1,Holidays!$A$2:$A$40)</f>
-        <v>46308</v>
+        <v>46318</v>
       </c>
       <c r="J27" s="47">
         <f>IF('Project Status'!E27="","",'Project Status'!E27)</f>
-        <v>46314</v>
-      </c>
-      <c r="K27" s="47" t="str">
+        <v>46319</v>
+      </c>
+      <c r="K27" s="47">
         <f>IF('Project Status'!F27="","",'Project Status'!F27)</f>
-        <v/>
+        <v>46319</v>
       </c>
       <c r="L27" s="45" t="str">
         <f>IF('Project Status'!G27="","",'Project Status'!G27)</f>
-        <v>In progress</v>
-      </c>
-      <c r="M27" s="45" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="M27" s="45">
         <f>IF(OR(K27="",I27=""),"",IF(K27&gt;=I27,NETWORKDAYS(I27,K27,Holidays!$A$2:$A$40)-1,-(NETWORKDAYS(K27,I27,Holidays!$A$2:$A$40)-1)))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N27" s="48" t="str">
         <f t="shared" ca="1" si="8"/>
@@ -8869,11 +8936,11 @@
       </c>
       <c r="AJ27" s="48" t="str">
         <f t="shared" ca="1" si="10"/>
-        <v>●</v>
+        <v/>
       </c>
       <c r="AK27" s="48" t="str">
         <f t="shared" ca="1" si="10"/>
-        <v>●</v>
+        <v/>
       </c>
       <c r="AL27" s="48" t="str">
         <f t="shared" ca="1" si="10"/>
@@ -8924,18 +8991,18 @@
         <v/>
       </c>
       <c r="AX27" s="49" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
     </row>
     <row r="28" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A28" s="45" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
       <c r="B28" s="45" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="C28" s="45" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="D28" s="46" t="s">
         <v>13</v>
@@ -8947,30 +9014,29 @@
         <v>2</v>
       </c>
       <c r="G28" s="45" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="H28" s="47">
-        <v>46310</v>
+        <v>46318</v>
       </c>
       <c r="I28" s="47">
-        <f>WORKDAY(H28,E28-1,Holidays!$A$2:$A$40)</f>
-        <v>46311</v>
-      </c>
-      <c r="J28" s="47" t="str">
+        <v>46318</v>
+      </c>
+      <c r="J28" s="47">
         <f>IF('Project Status'!E28="","",'Project Status'!E28)</f>
-        <v/>
-      </c>
-      <c r="K28" s="47" t="str">
+        <v>46319</v>
+      </c>
+      <c r="K28" s="47">
         <f>IF('Project Status'!F28="","",'Project Status'!F28)</f>
-        <v/>
+        <v>46319</v>
       </c>
       <c r="L28" s="45" t="str">
         <f>IF('Project Status'!G28="","",'Project Status'!G28)</f>
-        <v>Incident</v>
-      </c>
-      <c r="M28" s="45" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="M28" s="45">
         <f>IF(OR(K28="",I28=""),"",IF(K28&gt;=I28,NETWORKDAYS(I28,K28,Holidays!$A$2:$A$40)-1,-(NETWORKDAYS(K28,I28,Holidays!$A$2:$A$40)-1)))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N28" s="48" t="str">
         <f t="shared" ca="1" si="8"/>
@@ -9117,18 +9183,18 @@
         <v/>
       </c>
       <c r="AX28" s="49" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
     </row>
     <row r="29" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A29" s="45" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="B29" s="45" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="C29" s="45" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
       <c r="D29" s="52" t="s">
         <v>23</v>
@@ -9140,18 +9206,17 @@
         <v>3</v>
       </c>
       <c r="G29" s="45" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="H29" s="47">
-        <v>46308</v>
+        <v>46318</v>
       </c>
       <c r="I29" s="47">
-        <f>WORKDAY(H29,E29-1,Holidays!$A$2:$A$40)</f>
-        <v>46310</v>
-      </c>
-      <c r="J29" s="47" t="str">
+        <v>46319</v>
+      </c>
+      <c r="J29" s="47">
         <f>IF('Project Status'!E29="","",'Project Status'!E29)</f>
-        <v/>
+        <v>46318</v>
       </c>
       <c r="K29" s="47" t="str">
         <f>IF('Project Status'!F29="","",'Project Status'!F29)</f>
@@ -9159,7 +9224,7 @@
       </c>
       <c r="L29" s="45" t="str">
         <f>IF('Project Status'!G29="","",'Project Status'!G29)</f>
-        <v>Incident</v>
+        <v>In progress</v>
       </c>
       <c r="M29" s="45" t="str">
         <f>IF(OR(K29="",I29=""),"",IF(K29&gt;=I29,NETWORKDAYS(I29,K29,Holidays!$A$2:$A$40)-1,-(NETWORKDAYS(K29,I29,Holidays!$A$2:$A$40)-1)))</f>
@@ -9271,7 +9336,7 @@
       </c>
       <c r="AN29" s="48" t="str">
         <f t="shared" ca="1" si="10"/>
-        <v/>
+        <v>●</v>
       </c>
       <c r="AO29" s="48" t="str">
         <f t="shared" ca="1" si="10"/>
@@ -9310,18 +9375,18 @@
         <v/>
       </c>
       <c r="AX29" s="49" t="s">
-        <v>211</v>
+        <v>217</v>
       </c>
     </row>
     <row r="30" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A30" s="45" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="B30" s="45" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="C30" s="45" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="D30" s="46" t="s">
         <v>13</v>
@@ -9333,30 +9398,29 @@
         <v>1</v>
       </c>
       <c r="G30" s="45" t="s">
-        <v>202</v>
+        <v>208</v>
       </c>
       <c r="H30" s="47">
-        <v>46309</v>
+        <v>46318</v>
       </c>
       <c r="I30" s="47">
-        <f>WORKDAY(H30,E30-1,Holidays!$A$2:$A$40)</f>
-        <v>46309</v>
+        <v>46318</v>
       </c>
       <c r="J30" s="47">
         <f>IF('Project Status'!E30="","",'Project Status'!E30)</f>
-        <v>46314</v>
-      </c>
-      <c r="K30" s="47" t="str">
+        <v>46319</v>
+      </c>
+      <c r="K30" s="47">
         <f>IF('Project Status'!F30="","",'Project Status'!F30)</f>
-        <v/>
+        <v>46319</v>
       </c>
       <c r="L30" s="45" t="str">
         <f>IF('Project Status'!G30="","",'Project Status'!G30)</f>
-        <v>In progress</v>
-      </c>
-      <c r="M30" s="45" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="M30" s="45">
         <f>IF(OR(K30="",I30=""),"",IF(K30&gt;=I30,NETWORKDAYS(I30,K30,Holidays!$A$2:$A$40)-1,-(NETWORKDAYS(K30,I30,Holidays!$A$2:$A$40)-1)))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N30" s="48" t="str">
         <f t="shared" ca="1" si="8"/>
@@ -9448,11 +9512,11 @@
       </c>
       <c r="AJ30" s="48" t="str">
         <f t="shared" ca="1" si="10"/>
-        <v>●</v>
+        <v/>
       </c>
       <c r="AK30" s="48" t="str">
         <f t="shared" ca="1" si="10"/>
-        <v>●</v>
+        <v/>
       </c>
       <c r="AL30" s="48" t="str">
         <f t="shared" ca="1" si="10"/>
@@ -9503,18 +9567,18 @@
         <v/>
       </c>
       <c r="AX30" s="49" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
     </row>
     <row r="31" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A31" s="45" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="B31" s="45" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="C31" s="45" t="s">
-        <v>216</v>
+        <v>222</v>
       </c>
       <c r="D31" s="55" t="s">
         <v>39</v>
@@ -9526,18 +9590,17 @@
         <v>1</v>
       </c>
       <c r="G31" s="45" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="H31" s="47">
-        <v>46308</v>
+        <v>46318</v>
       </c>
       <c r="I31" s="47">
-        <f>WORKDAY(H31,E31-1,Holidays!$A$2:$A$40)</f>
-        <v>46308</v>
-      </c>
-      <c r="J31" s="47" t="str">
+        <v>46318</v>
+      </c>
+      <c r="J31" s="47">
         <f>IF('Project Status'!E31="","",'Project Status'!E31)</f>
-        <v/>
+        <v>46319</v>
       </c>
       <c r="K31" s="47" t="str">
         <f>IF('Project Status'!F31="","",'Project Status'!F31)</f>
@@ -9545,7 +9608,7 @@
       </c>
       <c r="L31" s="45" t="str">
         <f>IF('Project Status'!G31="","",'Project Status'!G31)</f>
-        <v>Incident</v>
+        <v>In progress</v>
       </c>
       <c r="M31" s="45" t="str">
         <f>IF(OR(K31="",I31=""),"",IF(K31&gt;=I31,NETWORKDAYS(I31,K31,Holidays!$A$2:$A$40)-1,-(NETWORKDAYS(K31,I31,Holidays!$A$2:$A$40)-1)))</f>
@@ -9696,18 +9759,18 @@
         <v/>
       </c>
       <c r="AX31" s="49" t="s">
-        <v>217</v>
+        <v>223</v>
       </c>
     </row>
     <row r="32" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A32" s="45" t="s">
-        <v>218</v>
+        <v>224</v>
       </c>
       <c r="B32" s="45" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="C32" s="45" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
       <c r="D32" s="46" t="s">
         <v>13</v>
@@ -9719,18 +9782,17 @@
         <v>1</v>
       </c>
       <c r="G32" s="45" t="s">
-        <v>220</v>
+        <v>226</v>
       </c>
       <c r="H32" s="47">
-        <v>46314</v>
+        <v>46319</v>
       </c>
       <c r="I32" s="47">
-        <f>WORKDAY(H32,E32-1,Holidays!$A$2:$A$40)</f>
-        <v>46314</v>
-      </c>
-      <c r="J32" s="47" t="str">
+        <v>46320</v>
+      </c>
+      <c r="J32" s="47">
         <f>IF('Project Status'!E32="","",'Project Status'!E32)</f>
-        <v/>
+        <v>46319</v>
       </c>
       <c r="K32" s="47" t="str">
         <f>IF('Project Status'!F32="","",'Project Status'!F32)</f>
@@ -9738,7 +9800,7 @@
       </c>
       <c r="L32" s="45" t="str">
         <f>IF('Project Status'!G32="","",'Project Status'!G32)</f>
-        <v>Incident</v>
+        <v>In progress</v>
       </c>
       <c r="M32" s="45" t="str">
         <f>IF(OR(K32="",I32=""),"",IF(K32&gt;=I32,NETWORKDAYS(I32,K32,Holidays!$A$2:$A$40)-1,-(NETWORKDAYS(K32,I32,Holidays!$A$2:$A$40)-1)))</f>
@@ -9889,18 +9951,18 @@
         <v/>
       </c>
       <c r="AX32" s="49" t="s">
-        <v>221</v>
+        <v>227</v>
       </c>
     </row>
     <row r="33" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A33" s="45" t="s">
-        <v>222</v>
+        <v>228</v>
       </c>
       <c r="B33" s="45" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="C33" s="45" t="s">
-        <v>223</v>
+        <v>229</v>
       </c>
       <c r="D33" s="50" t="s">
         <v>17</v>
@@ -9912,30 +9974,29 @@
         <v>1</v>
       </c>
       <c r="G33" s="45" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="H33" s="47">
-        <v>46309</v>
+        <v>46318</v>
       </c>
       <c r="I33" s="47">
-        <f>WORKDAY(H33,E33-1,Holidays!$A$2:$A$40)</f>
-        <v>46309</v>
-      </c>
-      <c r="J33" s="47" t="str">
+        <v>46318</v>
+      </c>
+      <c r="J33" s="47">
         <f>IF('Project Status'!E33="","",'Project Status'!E33)</f>
-        <v/>
-      </c>
-      <c r="K33" s="47" t="str">
+        <v>46319</v>
+      </c>
+      <c r="K33" s="47">
         <f>IF('Project Status'!F33="","",'Project Status'!F33)</f>
-        <v/>
+        <v>46319</v>
       </c>
       <c r="L33" s="45" t="str">
         <f>IF('Project Status'!G33="","",'Project Status'!G33)</f>
-        <v>Incident</v>
-      </c>
-      <c r="M33" s="45" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="M33" s="45">
         <f>IF(OR(K33="",I33=""),"",IF(K33&gt;=I33,NETWORKDAYS(I33,K33,Holidays!$A$2:$A$40)-1,-(NETWORKDAYS(K33,I33,Holidays!$A$2:$A$40)-1)))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N33" s="48" t="str">
         <f t="shared" ca="1" si="8"/>
@@ -10082,33 +10143,33 @@
         <v/>
       </c>
       <c r="AX33" s="49" t="s">
-        <v>224</v>
+        <v>230</v>
       </c>
     </row>
     <row r="34" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A34" s="29" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="B34" s="30" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="C34" s="30" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D34" s="30"/>
       <c r="E34" s="30">
         <f>NETWORKDAYS(H34,I34,Holidays!$A$2:$A$40)</f>
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F34" s="30"/>
       <c r="G34" s="30"/>
       <c r="H34" s="57">
         <f>MIN(H35:H43)</f>
-        <v>46309</v>
+        <v>46318</v>
       </c>
       <c r="I34" s="57">
         <f>MAX(I35:I43)</f>
-        <v>46316</v>
+        <v>46320</v>
       </c>
       <c r="J34" s="30"/>
       <c r="K34" s="30"/>
@@ -10153,13 +10214,13 @@
     </row>
     <row r="35" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A35" s="45" t="s">
-        <v>226</v>
+        <v>232</v>
       </c>
       <c r="B35" s="45" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="C35" s="45" t="s">
-        <v>227</v>
+        <v>233</v>
       </c>
       <c r="D35" s="54" t="s">
         <v>36</v>
@@ -10171,30 +10232,29 @@
         <v>1</v>
       </c>
       <c r="G35" s="45" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="H35" s="47">
-        <v>46310</v>
+        <v>46318</v>
       </c>
       <c r="I35" s="47">
-        <f>WORKDAY(H35,E35-1,Holidays!$A$2:$A$40)</f>
-        <v>46310</v>
+        <v>46318</v>
       </c>
       <c r="J35" s="47">
         <f>IF('Project Status'!E35="","",'Project Status'!E35)</f>
-        <v>46314</v>
-      </c>
-      <c r="K35" s="47" t="str">
+        <v>46318</v>
+      </c>
+      <c r="K35" s="47">
         <f>IF('Project Status'!F35="","",'Project Status'!F35)</f>
-        <v/>
+        <v>46319</v>
       </c>
       <c r="L35" s="45" t="str">
         <f>IF('Project Status'!G35="","",'Project Status'!G35)</f>
-        <v>In progress</v>
-      </c>
-      <c r="M35" s="45" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="M35" s="45">
         <f>IF(OR(K35="",I35=""),"",IF(K35&gt;=I35,NETWORKDAYS(I35,K35,Holidays!$A$2:$A$40)-1,-(NETWORKDAYS(K35,I35,Holidays!$A$2:$A$40)-1)))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N35" s="48" t="str">
         <f t="shared" ref="N35:W43" ca="1" si="12">IF(AND($J35&lt;&gt;"",N$4&gt;=$J35,N$4&lt;=IF($K35="",TODAY(),$K35),N$65=0),"●","")</f>
@@ -10286,11 +10346,11 @@
       </c>
       <c r="AJ35" s="48" t="str">
         <f t="shared" ca="1" si="14"/>
-        <v>●</v>
+        <v/>
       </c>
       <c r="AK35" s="48" t="str">
         <f t="shared" ca="1" si="14"/>
-        <v>●</v>
+        <v/>
       </c>
       <c r="AL35" s="48" t="str">
         <f t="shared" ca="1" si="14"/>
@@ -10302,7 +10362,7 @@
       </c>
       <c r="AN35" s="48" t="str">
         <f t="shared" ca="1" si="14"/>
-        <v/>
+        <v>●</v>
       </c>
       <c r="AO35" s="48" t="str">
         <f t="shared" ca="1" si="14"/>
@@ -10341,18 +10401,18 @@
         <v/>
       </c>
       <c r="AX35" s="49" t="s">
-        <v>228</v>
+        <v>234</v>
       </c>
     </row>
     <row r="36" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A36" s="45" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
       <c r="B36" s="45" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="C36" s="45" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
       <c r="D36" s="54" t="s">
         <v>36</v>
@@ -10364,30 +10424,29 @@
         <v>2</v>
       </c>
       <c r="G36" s="45" t="s">
-        <v>226</v>
+        <v>232</v>
       </c>
       <c r="H36" s="47">
-        <v>46311</v>
+        <v>46319</v>
       </c>
       <c r="I36" s="47">
-        <f>WORKDAY(H36,E36-1,Holidays!$A$2:$A$40)</f>
-        <v>46314</v>
-      </c>
-      <c r="J36" s="47" t="str">
+        <v>46319</v>
+      </c>
+      <c r="J36" s="47">
         <f>IF('Project Status'!E36="","",'Project Status'!E36)</f>
-        <v/>
-      </c>
-      <c r="K36" s="47" t="str">
+        <v>46319</v>
+      </c>
+      <c r="K36" s="47">
         <f>IF('Project Status'!F36="","",'Project Status'!F36)</f>
-        <v/>
+        <v>46319</v>
       </c>
       <c r="L36" s="45" t="str">
         <f>IF('Project Status'!G36="","",'Project Status'!G36)</f>
-        <v>Incident</v>
-      </c>
-      <c r="M36" s="45" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="M36" s="45">
         <f>IF(OR(K36="",I36=""),"",IF(K36&gt;=I36,NETWORKDAYS(I36,K36,Holidays!$A$2:$A$40)-1,-(NETWORKDAYS(K36,I36,Holidays!$A$2:$A$40)-1)))</f>
-        <v/>
+        <v>-1</v>
       </c>
       <c r="N36" s="48" t="str">
         <f t="shared" ca="1" si="12"/>
@@ -10534,18 +10593,18 @@
         <v/>
       </c>
       <c r="AX36" s="49" t="s">
-        <v>231</v>
+        <v>237</v>
       </c>
     </row>
     <row r="37" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A37" s="45" t="s">
-        <v>232</v>
+        <v>238</v>
       </c>
       <c r="B37" s="45" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="C37" s="45" t="s">
-        <v>233</v>
+        <v>239</v>
       </c>
       <c r="D37" s="55" t="s">
         <v>39</v>
@@ -10557,30 +10616,29 @@
         <v>2</v>
       </c>
       <c r="G37" s="45" t="s">
-        <v>234</v>
+        <v>240</v>
       </c>
       <c r="H37" s="47">
-        <v>46309</v>
+        <v>46318</v>
       </c>
       <c r="I37" s="47">
-        <f>WORKDAY(H37,E37-1,Holidays!$A$2:$A$40)</f>
-        <v>46310</v>
-      </c>
-      <c r="J37" s="47" t="str">
+        <v>46318</v>
+      </c>
+      <c r="J37" s="47">
         <f>IF('Project Status'!E37="","",'Project Status'!E37)</f>
-        <v/>
-      </c>
-      <c r="K37" s="47" t="str">
+        <v>46319</v>
+      </c>
+      <c r="K37" s="47">
         <f>IF('Project Status'!F37="","",'Project Status'!F37)</f>
-        <v/>
+        <v>46319</v>
       </c>
       <c r="L37" s="45" t="str">
         <f>IF('Project Status'!G37="","",'Project Status'!G37)</f>
-        <v>Incident</v>
-      </c>
-      <c r="M37" s="45" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="M37" s="45">
         <f>IF(OR(K37="",I37=""),"",IF(K37&gt;=I37,NETWORKDAYS(I37,K37,Holidays!$A$2:$A$40)-1,-(NETWORKDAYS(K37,I37,Holidays!$A$2:$A$40)-1)))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N37" s="48" t="str">
         <f t="shared" ca="1" si="12"/>
@@ -10727,18 +10785,18 @@
         <v/>
       </c>
       <c r="AX37" s="49" t="s">
-        <v>235</v>
+        <v>241</v>
       </c>
     </row>
     <row r="38" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A38" s="45" t="s">
-        <v>236</v>
+        <v>242</v>
       </c>
       <c r="B38" s="45" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="C38" s="45" t="s">
-        <v>237</v>
+        <v>243</v>
       </c>
       <c r="D38" s="55" t="s">
         <v>39</v>
@@ -10750,30 +10808,29 @@
         <v>2</v>
       </c>
       <c r="G38" s="45" t="s">
-        <v>232</v>
+        <v>238</v>
       </c>
       <c r="H38" s="47">
-        <v>46311</v>
+        <v>46319</v>
       </c>
       <c r="I38" s="47">
-        <f>WORKDAY(H38,E38-1,Holidays!$A$2:$A$40)</f>
-        <v>46314</v>
-      </c>
-      <c r="J38" s="47" t="str">
+        <v>46319</v>
+      </c>
+      <c r="J38" s="47">
         <f>IF('Project Status'!E38="","",'Project Status'!E38)</f>
-        <v/>
-      </c>
-      <c r="K38" s="47" t="str">
+        <v>46319</v>
+      </c>
+      <c r="K38" s="47">
         <f>IF('Project Status'!F38="","",'Project Status'!F38)</f>
-        <v/>
+        <v>46319</v>
       </c>
       <c r="L38" s="45" t="str">
         <f>IF('Project Status'!G38="","",'Project Status'!G38)</f>
-        <v>Incident</v>
-      </c>
-      <c r="M38" s="45" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="M38" s="45">
         <f>IF(OR(K38="",I38=""),"",IF(K38&gt;=I38,NETWORKDAYS(I38,K38,Holidays!$A$2:$A$40)-1,-(NETWORKDAYS(K38,I38,Holidays!$A$2:$A$40)-1)))</f>
-        <v/>
+        <v>-1</v>
       </c>
       <c r="N38" s="48" t="str">
         <f t="shared" ca="1" si="12"/>
@@ -10920,18 +10977,18 @@
         <v/>
       </c>
       <c r="AX38" s="49" t="s">
-        <v>238</v>
+        <v>244</v>
       </c>
     </row>
     <row r="39" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A39" s="45" t="s">
-        <v>239</v>
+        <v>245</v>
       </c>
       <c r="B39" s="45" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="C39" s="45" t="s">
-        <v>240</v>
+        <v>246</v>
       </c>
       <c r="D39" s="55" t="s">
         <v>39</v>
@@ -10943,18 +11000,17 @@
         <v>1</v>
       </c>
       <c r="G39" s="45" t="s">
-        <v>241</v>
+        <v>247</v>
       </c>
       <c r="H39" s="47">
-        <v>46315</v>
+        <v>46319</v>
       </c>
       <c r="I39" s="47">
-        <f>WORKDAY(H39,E39-1,Holidays!$A$2:$A$40)</f>
-        <v>46315</v>
-      </c>
-      <c r="J39" s="47" t="str">
+        <v>46319</v>
+      </c>
+      <c r="J39" s="47">
         <f>IF('Project Status'!E39="","",'Project Status'!E39)</f>
-        <v/>
+        <v>46319</v>
       </c>
       <c r="K39" s="47" t="str">
         <f>IF('Project Status'!F39="","",'Project Status'!F39)</f>
@@ -10962,7 +11018,7 @@
       </c>
       <c r="L39" s="45" t="str">
         <f>IF('Project Status'!G39="","",'Project Status'!G39)</f>
-        <v>Pending</v>
+        <v>In progress</v>
       </c>
       <c r="M39" s="45" t="str">
         <f>IF(OR(K39="",I39=""),"",IF(K39&gt;=I39,NETWORKDAYS(I39,K39,Holidays!$A$2:$A$40)-1,-(NETWORKDAYS(K39,I39,Holidays!$A$2:$A$40)-1)))</f>
@@ -11113,18 +11169,18 @@
         <v/>
       </c>
       <c r="AX39" s="49" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
     </row>
     <row r="40" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A40" s="45" t="s">
-        <v>243</v>
+        <v>249</v>
       </c>
       <c r="B40" s="45" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="C40" s="45" t="s">
-        <v>244</v>
+        <v>250</v>
       </c>
       <c r="D40" s="52" t="s">
         <v>23</v>
@@ -11136,14 +11192,13 @@
         <v>1</v>
       </c>
       <c r="G40" s="45" t="s">
-        <v>245</v>
+        <v>251</v>
       </c>
       <c r="H40" s="47">
-        <v>46314</v>
+        <v>46319</v>
       </c>
       <c r="I40" s="47">
-        <f>WORKDAY(H40,E40-1,Holidays!$A$2:$A$40)</f>
-        <v>46314</v>
+        <v>46319</v>
       </c>
       <c r="J40" s="47" t="str">
         <f>IF('Project Status'!E40="","",'Project Status'!E40)</f>
@@ -11155,7 +11210,7 @@
       </c>
       <c r="L40" s="45" t="str">
         <f>IF('Project Status'!G40="","",'Project Status'!G40)</f>
-        <v>Incident</v>
+        <v>Pending</v>
       </c>
       <c r="M40" s="45" t="str">
         <f>IF(OR(K40="",I40=""),"",IF(K40&gt;=I40,NETWORKDAYS(I40,K40,Holidays!$A$2:$A$40)-1,-(NETWORKDAYS(K40,I40,Holidays!$A$2:$A$40)-1)))</f>
@@ -11306,18 +11361,18 @@
         <v/>
       </c>
       <c r="AX40" s="49" t="s">
-        <v>246</v>
+        <v>252</v>
       </c>
     </row>
     <row r="41" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A41" s="45" t="s">
-        <v>247</v>
+        <v>253</v>
       </c>
       <c r="B41" s="45" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="C41" s="45" t="s">
-        <v>248</v>
+        <v>254</v>
       </c>
       <c r="D41" s="52" t="s">
         <v>23</v>
@@ -11329,14 +11384,13 @@
         <v>1</v>
       </c>
       <c r="G41" s="45" t="s">
-        <v>243</v>
+        <v>249</v>
       </c>
       <c r="H41" s="47">
-        <v>46315</v>
+        <v>46319</v>
       </c>
       <c r="I41" s="47">
-        <f>WORKDAY(H41,E41-1,Holidays!$A$2:$A$40)</f>
-        <v>46315</v>
+        <v>46319</v>
       </c>
       <c r="J41" s="47" t="str">
         <f>IF('Project Status'!E41="","",'Project Status'!E41)</f>
@@ -11499,18 +11553,18 @@
         <v/>
       </c>
       <c r="AX41" s="49" t="s">
-        <v>249</v>
+        <v>255</v>
       </c>
     </row>
     <row r="42" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A42" s="45" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="B42" s="45" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="C42" s="45" t="s">
-        <v>251</v>
+        <v>257</v>
       </c>
       <c r="D42" s="50" t="s">
         <v>17</v>
@@ -11522,14 +11576,13 @@
         <v>1</v>
       </c>
       <c r="G42" s="45" t="s">
-        <v>252</v>
+        <v>258</v>
       </c>
       <c r="H42" s="47">
-        <v>46316</v>
+        <v>46320</v>
       </c>
       <c r="I42" s="47">
-        <f>WORKDAY(H42,E42-1,Holidays!$A$2:$A$40)</f>
-        <v>46316</v>
+        <v>46320</v>
       </c>
       <c r="J42" s="47" t="str">
         <f>IF('Project Status'!E42="","",'Project Status'!E42)</f>
@@ -11692,18 +11745,18 @@
         <v/>
       </c>
       <c r="AX42" s="49" t="s">
-        <v>253</v>
+        <v>259</v>
       </c>
     </row>
     <row r="43" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A43" s="45" t="s">
-        <v>254</v>
+        <v>260</v>
       </c>
       <c r="B43" s="45" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="C43" s="45" t="s">
-        <v>255</v>
+        <v>261</v>
       </c>
       <c r="D43" s="46" t="s">
         <v>13</v>
@@ -11715,30 +11768,29 @@
         <v>1</v>
       </c>
       <c r="G43" s="45" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
       <c r="H43" s="47">
-        <v>46315</v>
+        <v>46319</v>
       </c>
       <c r="I43" s="47">
-        <f>WORKDAY(H43,E43-1,Holidays!$A$2:$A$40)</f>
-        <v>46315</v>
-      </c>
-      <c r="J43" s="47" t="str">
+        <v>46319</v>
+      </c>
+      <c r="J43" s="47">
         <f>IF('Project Status'!E43="","",'Project Status'!E43)</f>
-        <v/>
-      </c>
-      <c r="K43" s="47" t="str">
+        <v>46319</v>
+      </c>
+      <c r="K43" s="47">
         <f>IF('Project Status'!F43="","",'Project Status'!F43)</f>
-        <v/>
+        <v>46319</v>
       </c>
       <c r="L43" s="45" t="str">
         <f>IF('Project Status'!G43="","",'Project Status'!G43)</f>
-        <v>Pending</v>
-      </c>
-      <c r="M43" s="45" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="M43" s="45">
         <f>IF(OR(K43="",I43=""),"",IF(K43&gt;=I43,NETWORKDAYS(I43,K43,Holidays!$A$2:$A$40)-1,-(NETWORKDAYS(K43,I43,Holidays!$A$2:$A$40)-1)))</f>
-        <v/>
+        <v>-1</v>
       </c>
       <c r="N43" s="48" t="str">
         <f t="shared" ca="1" si="12"/>
@@ -11885,29 +11937,29 @@
         <v/>
       </c>
       <c r="AX43" s="49" t="s">
-        <v>256</v>
+        <v>262</v>
       </c>
     </row>
     <row r="44" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A44" s="31" t="s">
-        <v>257</v>
+        <v>263</v>
       </c>
       <c r="B44" s="32" t="s">
-        <v>257</v>
+        <v>263</v>
       </c>
       <c r="C44" s="32" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="D44" s="32"/>
       <c r="E44" s="32">
         <f>NETWORKDAYS(H44,I44,Holidays!$A$2:$A$40)</f>
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="F44" s="32"/>
       <c r="G44" s="32"/>
       <c r="H44" s="58">
         <f>MIN(H45:H60)</f>
-        <v>46315</v>
+        <v>46319</v>
       </c>
       <c r="I44" s="58">
         <f>MAX(I45:I60)</f>
@@ -11956,13 +12008,13 @@
     </row>
     <row r="45" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A45" s="45" t="s">
-        <v>258</v>
+        <v>264</v>
       </c>
       <c r="B45" s="45" t="s">
-        <v>257</v>
+        <v>263</v>
       </c>
       <c r="C45" s="45" t="s">
-        <v>259</v>
+        <v>265</v>
       </c>
       <c r="D45" s="52" t="s">
         <v>23</v>
@@ -11974,18 +12026,17 @@
         <v>2</v>
       </c>
       <c r="G45" s="45" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="H45" s="47">
-        <v>46316</v>
+        <v>46319</v>
       </c>
       <c r="I45" s="47">
-        <f>WORKDAY(H45,E45-1,Holidays!$A$2:$A$40)</f>
-        <v>46317</v>
-      </c>
-      <c r="J45" s="47" t="str">
+        <v>46319</v>
+      </c>
+      <c r="J45" s="47">
         <f>IF('Project Status'!E45="","",'Project Status'!E45)</f>
-        <v/>
+        <v>46319</v>
       </c>
       <c r="K45" s="47" t="str">
         <f>IF('Project Status'!F45="","",'Project Status'!F45)</f>
@@ -11993,7 +12044,7 @@
       </c>
       <c r="L45" s="45" t="str">
         <f>IF('Project Status'!G45="","",'Project Status'!G45)</f>
-        <v>Pending</v>
+        <v>In progress</v>
       </c>
       <c r="M45" s="45" t="str">
         <f>IF(OR(K45="",I45=""),"",IF(K45&gt;=I45,NETWORKDAYS(I45,K45,Holidays!$A$2:$A$40)-1,-(NETWORKDAYS(K45,I45,Holidays!$A$2:$A$40)-1)))</f>
@@ -12144,18 +12195,18 @@
         <v/>
       </c>
       <c r="AX45" s="49" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
     </row>
     <row r="46" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A46" s="45" t="s">
-        <v>261</v>
+        <v>267</v>
       </c>
       <c r="B46" s="45" t="s">
-        <v>257</v>
+        <v>263</v>
       </c>
       <c r="C46" s="45" t="s">
-        <v>262</v>
+        <v>268</v>
       </c>
       <c r="D46" s="46" t="s">
         <v>13</v>
@@ -12167,14 +12218,13 @@
         <v>2</v>
       </c>
       <c r="G46" s="45" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
       <c r="H46" s="47">
-        <v>46316</v>
+        <v>46320</v>
       </c>
       <c r="I46" s="47">
-        <f>WORKDAY(H46,E46-1,Holidays!$A$2:$A$40)</f>
-        <v>46317</v>
+        <v>46320</v>
       </c>
       <c r="J46" s="47" t="str">
         <f>IF('Project Status'!E46="","",'Project Status'!E46)</f>
@@ -12337,18 +12387,18 @@
         <v/>
       </c>
       <c r="AX46" s="49" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
     </row>
     <row r="47" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A47" s="45" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="B47" s="45" t="s">
-        <v>257</v>
+        <v>263</v>
       </c>
       <c r="C47" s="45" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="D47" s="54" t="s">
         <v>36</v>
@@ -12360,14 +12410,13 @@
         <v>2</v>
       </c>
       <c r="G47" s="45" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
       <c r="H47" s="47">
-        <v>46315</v>
+        <v>46320</v>
       </c>
       <c r="I47" s="47">
-        <f>WORKDAY(H47,E47-1,Holidays!$A$2:$A$40)</f>
-        <v>46316</v>
+        <v>46320</v>
       </c>
       <c r="J47" s="47" t="str">
         <f>IF('Project Status'!E47="","",'Project Status'!E47)</f>
@@ -12530,18 +12579,18 @@
         <v/>
       </c>
       <c r="AX47" s="49" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
     </row>
     <row r="48" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A48" s="45" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="B48" s="45" t="s">
-        <v>257</v>
+        <v>263</v>
       </c>
       <c r="C48" s="45" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="D48" s="55" t="s">
         <v>39</v>
@@ -12553,14 +12602,13 @@
         <v>2</v>
       </c>
       <c r="G48" s="45" t="s">
-        <v>239</v>
+        <v>245</v>
       </c>
       <c r="H48" s="47">
-        <v>46316</v>
+        <v>46320</v>
       </c>
       <c r="I48" s="47">
-        <f>WORKDAY(H48,E48-1,Holidays!$A$2:$A$40)</f>
-        <v>46317</v>
+        <v>46320</v>
       </c>
       <c r="J48" s="47" t="str">
         <f>IF('Project Status'!E48="","",'Project Status'!E48)</f>
@@ -12723,18 +12771,18 @@
         <v/>
       </c>
       <c r="AX48" s="49" t="s">
-        <v>270</v>
+        <v>276</v>
       </c>
     </row>
     <row r="49" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A49" s="45" t="s">
-        <v>271</v>
+        <v>277</v>
       </c>
       <c r="B49" s="45" t="s">
-        <v>257</v>
+        <v>263</v>
       </c>
       <c r="C49" s="45" t="s">
-        <v>272</v>
+        <v>278</v>
       </c>
       <c r="D49" s="50" t="s">
         <v>17</v>
@@ -12746,14 +12794,13 @@
         <v>2</v>
       </c>
       <c r="G49" s="45" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="H49" s="47">
-        <v>46317</v>
+        <v>46320</v>
       </c>
       <c r="I49" s="47">
-        <f>WORKDAY(H49,E49-1,Holidays!$A$2:$A$40)</f>
-        <v>46318</v>
+        <v>46320</v>
       </c>
       <c r="J49" s="47" t="str">
         <f>IF('Project Status'!E49="","",'Project Status'!E49)</f>
@@ -12916,18 +12963,18 @@
         <v/>
       </c>
       <c r="AX49" s="49" t="s">
-        <v>273</v>
+        <v>279</v>
       </c>
     </row>
     <row r="50" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A50" s="45" t="s">
-        <v>196</v>
+        <v>202</v>
       </c>
       <c r="B50" s="45" t="s">
-        <v>257</v>
+        <v>263</v>
       </c>
       <c r="C50" s="45" t="s">
-        <v>274</v>
+        <v>280</v>
       </c>
       <c r="D50" s="52" t="s">
         <v>23</v>
@@ -12939,13 +12986,12 @@
         <v>1</v>
       </c>
       <c r="G50" s="45" t="s">
-        <v>275</v>
+        <v>281</v>
       </c>
       <c r="H50" s="47">
         <v>46321</v>
       </c>
       <c r="I50" s="47">
-        <f>WORKDAY(H50,E50-1,Holidays!$A$2:$A$40)</f>
         <v>46321</v>
       </c>
       <c r="J50" s="47" t="str">
@@ -13109,18 +13155,18 @@
         <v/>
       </c>
       <c r="AX50" s="49" t="s">
-        <v>276</v>
+        <v>282</v>
       </c>
     </row>
     <row r="51" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A51" s="45" t="s">
-        <v>277</v>
+        <v>283</v>
       </c>
       <c r="B51" s="45" t="s">
-        <v>257</v>
+        <v>263</v>
       </c>
       <c r="C51" s="45" t="s">
-        <v>278</v>
+        <v>284</v>
       </c>
       <c r="D51" s="54" t="s">
         <v>36</v>
@@ -13132,14 +13178,13 @@
         <v>1</v>
       </c>
       <c r="G51" s="45" t="s">
-        <v>196</v>
+        <v>202</v>
       </c>
       <c r="H51" s="47">
-        <v>46322</v>
+        <v>46321</v>
       </c>
       <c r="I51" s="47">
-        <f>WORKDAY(H51,E51-1,Holidays!$A$2:$A$40)</f>
-        <v>46322</v>
+        <v>46321</v>
       </c>
       <c r="J51" s="47" t="str">
         <f>IF('Project Status'!E51="","",'Project Status'!E51)</f>
@@ -13302,18 +13347,18 @@
         <v/>
       </c>
       <c r="AX51" s="49" t="s">
-        <v>279</v>
+        <v>285</v>
       </c>
     </row>
     <row r="52" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A52" s="45" t="s">
-        <v>280</v>
+        <v>286</v>
       </c>
       <c r="B52" s="45" t="s">
-        <v>257</v>
+        <v>263</v>
       </c>
       <c r="C52" s="45" t="s">
-        <v>281</v>
+        <v>287</v>
       </c>
       <c r="D52" s="46" t="s">
         <v>13</v>
@@ -13325,14 +13370,13 @@
         <v>1</v>
       </c>
       <c r="G52" s="45" t="s">
-        <v>196</v>
+        <v>202</v>
       </c>
       <c r="H52" s="47">
-        <v>46322</v>
+        <v>46321</v>
       </c>
       <c r="I52" s="47">
-        <f>WORKDAY(H52,E52-1,Holidays!$A$2:$A$40)</f>
-        <v>46322</v>
+        <v>46321</v>
       </c>
       <c r="J52" s="47" t="str">
         <f>IF('Project Status'!E52="","",'Project Status'!E52)</f>
@@ -13495,18 +13539,18 @@
         <v/>
       </c>
       <c r="AX52" s="49" t="s">
-        <v>282</v>
+        <v>288</v>
       </c>
     </row>
     <row r="53" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A53" s="45" t="s">
-        <v>283</v>
+        <v>289</v>
       </c>
       <c r="B53" s="45" t="s">
-        <v>257</v>
+        <v>263</v>
       </c>
       <c r="C53" s="45" t="s">
-        <v>284</v>
+        <v>290</v>
       </c>
       <c r="D53" s="52" t="s">
         <v>23</v>
@@ -13518,14 +13562,13 @@
         <v>1</v>
       </c>
       <c r="G53" s="45" t="s">
-        <v>285</v>
+        <v>291</v>
       </c>
       <c r="H53" s="47">
-        <v>46323</v>
+        <v>46321</v>
       </c>
       <c r="I53" s="47">
-        <f>WORKDAY(H53,E53-1,Holidays!$A$2:$A$40)</f>
-        <v>46323</v>
+        <v>46321</v>
       </c>
       <c r="J53" s="47" t="str">
         <f>IF('Project Status'!E53="","",'Project Status'!E53)</f>
@@ -13688,18 +13731,18 @@
         <v/>
       </c>
       <c r="AX53" s="49" t="s">
-        <v>286</v>
+        <v>292</v>
       </c>
     </row>
     <row r="54" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A54" s="45" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
       <c r="B54" s="45" t="s">
-        <v>257</v>
+        <v>263</v>
       </c>
       <c r="C54" s="45" t="s">
-        <v>288</v>
+        <v>294</v>
       </c>
       <c r="D54" s="52" t="s">
         <v>23</v>
@@ -13711,14 +13754,13 @@
         <v>1</v>
       </c>
       <c r="G54" s="45" t="s">
-        <v>283</v>
+        <v>289</v>
       </c>
       <c r="H54" s="47">
-        <v>46324</v>
+        <v>46322</v>
       </c>
       <c r="I54" s="47">
-        <f>WORKDAY(H54,E54-1,Holidays!$A$2:$A$40)</f>
-        <v>46324</v>
+        <v>46322</v>
       </c>
       <c r="J54" s="47" t="str">
         <f>IF('Project Status'!E54="","",'Project Status'!E54)</f>
@@ -13881,18 +13923,18 @@
         <v/>
       </c>
       <c r="AX54" s="49" t="s">
-        <v>289</v>
+        <v>295</v>
       </c>
     </row>
     <row r="55" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A55" s="45" t="s">
-        <v>290</v>
+        <v>296</v>
       </c>
       <c r="B55" s="45" t="s">
-        <v>257</v>
+        <v>263</v>
       </c>
       <c r="C55" s="45" t="s">
-        <v>291</v>
+        <v>297</v>
       </c>
       <c r="D55" s="46" t="s">
         <v>13</v>
@@ -13904,14 +13946,13 @@
         <v>1</v>
       </c>
       <c r="G55" s="45" t="s">
-        <v>283</v>
+        <v>289</v>
       </c>
       <c r="H55" s="47">
-        <v>46324</v>
+        <v>46322</v>
       </c>
       <c r="I55" s="47">
-        <f>WORKDAY(H55,E55-1,Holidays!$A$2:$A$40)</f>
-        <v>46324</v>
+        <v>46322</v>
       </c>
       <c r="J55" s="47" t="str">
         <f>IF('Project Status'!E55="","",'Project Status'!E55)</f>
@@ -14074,18 +14115,18 @@
         <v/>
       </c>
       <c r="AX55" s="49" t="s">
-        <v>292</v>
+        <v>298</v>
       </c>
     </row>
     <row r="56" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A56" s="45" t="s">
-        <v>293</v>
+        <v>299</v>
       </c>
       <c r="B56" s="45" t="s">
-        <v>257</v>
+        <v>263</v>
       </c>
       <c r="C56" s="45" t="s">
-        <v>294</v>
+        <v>300</v>
       </c>
       <c r="D56" s="50" t="s">
         <v>17</v>
@@ -14097,14 +14138,13 @@
         <v>1</v>
       </c>
       <c r="G56" s="45" t="s">
-        <v>283</v>
+        <v>289</v>
       </c>
       <c r="H56" s="47">
-        <v>46324</v>
+        <v>46322</v>
       </c>
       <c r="I56" s="47">
-        <f>WORKDAY(H56,E56-1,Holidays!$A$2:$A$40)</f>
-        <v>46324</v>
+        <v>46322</v>
       </c>
       <c r="J56" s="47" t="str">
         <f>IF('Project Status'!E56="","",'Project Status'!E56)</f>
@@ -14267,18 +14307,18 @@
         <v/>
       </c>
       <c r="AX56" s="49" t="s">
-        <v>295</v>
+        <v>301</v>
       </c>
     </row>
     <row r="57" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A57" s="45" t="s">
-        <v>296</v>
+        <v>302</v>
       </c>
       <c r="B57" s="45" t="s">
-        <v>257</v>
+        <v>263</v>
       </c>
       <c r="C57" s="45" t="s">
-        <v>297</v>
+        <v>303</v>
       </c>
       <c r="D57" s="54" t="s">
         <v>36</v>
@@ -14290,14 +14330,13 @@
         <v>1</v>
       </c>
       <c r="G57" s="45" t="s">
-        <v>283</v>
+        <v>289</v>
       </c>
       <c r="H57" s="47">
-        <v>46324</v>
+        <v>46322</v>
       </c>
       <c r="I57" s="47">
-        <f>WORKDAY(H57,E57-1,Holidays!$A$2:$A$40)</f>
-        <v>46324</v>
+        <v>46322</v>
       </c>
       <c r="J57" s="47" t="str">
         <f>IF('Project Status'!E57="","",'Project Status'!E57)</f>
@@ -14460,18 +14499,18 @@
         <v/>
       </c>
       <c r="AX57" s="49" t="s">
-        <v>298</v>
+        <v>304</v>
       </c>
     </row>
     <row r="58" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A58" s="45" t="s">
-        <v>299</v>
+        <v>305</v>
       </c>
       <c r="B58" s="45" t="s">
-        <v>257</v>
+        <v>263</v>
       </c>
       <c r="C58" s="45" t="s">
-        <v>300</v>
+        <v>306</v>
       </c>
       <c r="D58" s="55" t="s">
         <v>39</v>
@@ -14483,14 +14522,13 @@
         <v>1</v>
       </c>
       <c r="G58" s="45" t="s">
-        <v>283</v>
+        <v>289</v>
       </c>
       <c r="H58" s="47">
-        <v>46324</v>
+        <v>46322</v>
       </c>
       <c r="I58" s="47">
-        <f>WORKDAY(H58,E58-1,Holidays!$A$2:$A$40)</f>
-        <v>46324</v>
+        <v>46322</v>
       </c>
       <c r="J58" s="47" t="str">
         <f>IF('Project Status'!E58="","",'Project Status'!E58)</f>
@@ -14653,18 +14691,18 @@
         <v/>
       </c>
       <c r="AX58" s="49" t="s">
-        <v>301</v>
+        <v>307</v>
       </c>
     </row>
     <row r="59" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A59" s="45" t="s">
-        <v>302</v>
+        <v>308</v>
       </c>
       <c r="B59" s="45" t="s">
-        <v>257</v>
+        <v>263</v>
       </c>
       <c r="C59" s="45" t="s">
-        <v>303</v>
+        <v>309</v>
       </c>
       <c r="D59" s="46" t="s">
         <v>13</v>
@@ -14676,13 +14714,12 @@
         <v>1</v>
       </c>
       <c r="G59" s="45" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="H59" s="47">
         <v>46325</v>
       </c>
       <c r="I59" s="47">
-        <f>WORKDAY(H59,E59-1,Holidays!$A$2:$A$40)</f>
         <v>46325</v>
       </c>
       <c r="J59" s="47" t="str">
@@ -14846,18 +14883,18 @@
         <v/>
       </c>
       <c r="AX59" s="49" t="s">
-        <v>305</v>
+        <v>311</v>
       </c>
     </row>
     <row r="60" spans="1:50" x14ac:dyDescent="0.2">
       <c r="A60" s="45" t="s">
-        <v>306</v>
+        <v>312</v>
       </c>
       <c r="B60" s="45" t="s">
-        <v>257</v>
+        <v>263</v>
       </c>
       <c r="C60" s="45" t="s">
-        <v>307</v>
+        <v>313</v>
       </c>
       <c r="D60" s="54" t="s">
         <v>36</v>
@@ -14869,13 +14906,12 @@
         <v>2</v>
       </c>
       <c r="G60" s="45" t="s">
-        <v>302</v>
+        <v>308</v>
       </c>
       <c r="H60" s="47">
         <v>46328</v>
       </c>
       <c r="I60" s="47">
-        <f>WORKDAY(H60,E60-1,Holidays!$A$2:$A$40)</f>
         <v>46329</v>
       </c>
       <c r="J60" s="47" t="str">
@@ -15039,84 +15075,84 @@
         <v/>
       </c>
       <c r="AX60" s="49" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
     </row>
     <row r="62" spans="1:50" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C62" s="59" t="s">
-        <v>309</v>
+        <v>315</v>
       </c>
       <c r="N62" s="60" t="s">
-        <v>310</v>
+        <v>316</v>
       </c>
       <c r="AD62" s="60" t="s">
-        <v>311</v>
+        <v>317</v>
       </c>
       <c r="AJ62" s="60" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
       <c r="AL62" s="60" t="s">
-        <v>313</v>
+        <v>319</v>
       </c>
       <c r="AM62" s="60" t="s">
-        <v>314</v>
+        <v>320</v>
       </c>
       <c r="AO62" s="60" t="s">
-        <v>315</v>
+        <v>321</v>
       </c>
       <c r="AQ62" s="60" t="s">
-        <v>316</v>
+        <v>322</v>
       </c>
       <c r="AW62" s="60" t="s">
-        <v>317</v>
+        <v>323</v>
       </c>
     </row>
     <row r="63" spans="1:50" x14ac:dyDescent="0.2">
       <c r="C63" s="33" t="s">
-        <v>318</v>
+        <v>324</v>
       </c>
       <c r="N63" s="61" t="s">
-        <v>319</v>
+        <v>325</v>
       </c>
       <c r="P63" s="61" t="s">
-        <v>320</v>
+        <v>326</v>
       </c>
       <c r="U63" s="61" t="s">
-        <v>321</v>
+        <v>327</v>
       </c>
       <c r="X63" s="61" t="s">
-        <v>322</v>
+        <v>328</v>
       </c>
       <c r="Z63" s="61" t="s">
-        <v>323</v>
+        <v>329</v>
       </c>
       <c r="AC63" s="61" t="s">
-        <v>324</v>
+        <v>330</v>
       </c>
       <c r="AH63" s="61" t="s">
-        <v>325</v>
+        <v>331</v>
       </c>
       <c r="AJ63" s="61" t="s">
-        <v>326</v>
+        <v>332</v>
       </c>
       <c r="AM63" s="61" t="s">
-        <v>327</v>
+        <v>333</v>
       </c>
       <c r="AO63" s="61" t="s">
-        <v>328</v>
+        <v>334</v>
       </c>
       <c r="AW63" s="61" t="s">
-        <v>329</v>
+        <v>335</v>
       </c>
     </row>
     <row r="64" spans="1:50" x14ac:dyDescent="0.2">
       <c r="C64" s="62" t="s">
-        <v>330</v>
+        <v>336</v>
       </c>
     </row>
     <row r="65" spans="3:49" hidden="1" x14ac:dyDescent="0.2">
       <c r="C65" t="s">
-        <v>331</v>
+        <v>337</v>
       </c>
       <c r="N65">
         <f>IF(COUNTIF(Holidays!$A$2:$A$40,N$4)&gt;0,1,0)</f>
@@ -15271,8 +15307,8 @@
     <mergeCell ref="AJ3:AN3"/>
     <mergeCell ref="Z3:AD3"/>
     <mergeCell ref="N3:O3"/>
+    <mergeCell ref="P3:T3"/>
     <mergeCell ref="AO3:AS3"/>
-    <mergeCell ref="P3:T3"/>
     <mergeCell ref="AE3:AI3"/>
   </mergeCells>
   <conditionalFormatting sqref="L5:L60">
@@ -15450,24 +15486,24 @@
   <sheetData>
     <row r="1" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="63" t="s">
-        <v>332</v>
+        <v>338</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="11" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>333</v>
+        <v>339</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>334</v>
+        <v>340</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>335</v>
+        <v>341</v>
       </c>
       <c r="E3" s="11" t="s">
-        <v>336</v>
+        <v>342</v>
       </c>
       <c r="F3" s="11" t="s">
         <v>14</v>
@@ -15476,10 +15512,10 @@
         <v>46</v>
       </c>
       <c r="H3" s="11" t="s">
-        <v>337</v>
+        <v>343</v>
       </c>
       <c r="I3" s="80" t="s">
-        <v>338</v>
+        <v>344</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
@@ -15487,10 +15523,10 @@
         <v>23</v>
       </c>
       <c r="B4" s="65" t="s">
-        <v>339</v>
+        <v>345</v>
       </c>
       <c r="C4" s="65" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="D4" s="65">
         <f>COUNTIFS(Tasks!$D$5:$D$60,A4,Tasks!$B$5:$B$60,"&lt;&gt;P0",Tasks!$A$5:$A$60,"&lt;&gt;WP*")</f>
@@ -15506,14 +15542,14 @@
       </c>
       <c r="G4" s="65">
         <f>COUNTIFS(Tasks!$D$5:$D$60,A4,Tasks!$L$5:$L$60,"In progress")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H4" s="65">
         <f>COUNTIFS(Tasks!$D$5:$D$60,A4,Tasks!$L$5:$L$60,"Incident")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I4" t="s">
-        <v>341</v>
+        <v>347</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
@@ -15521,10 +15557,10 @@
         <v>36</v>
       </c>
       <c r="B5" s="65" t="s">
-        <v>342</v>
+        <v>348</v>
       </c>
       <c r="C5" s="65" t="s">
-        <v>343</v>
+        <v>349</v>
       </c>
       <c r="D5" s="65">
         <f>COUNTIFS(Tasks!$D$5:$D$60,A5,Tasks!$B$5:$B$60,"&lt;&gt;P0",Tasks!$A$5:$A$60,"&lt;&gt;WP*")</f>
@@ -15536,18 +15572,18 @@
       </c>
       <c r="F5" s="65">
         <f>COUNTIFS(Tasks!$D$5:$D$60,A5,Tasks!$L$5:$L$60,"Completed",Tasks!$B$5:$B$60,"&lt;&gt;P0")</f>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G5" s="65">
         <f>COUNTIFS(Tasks!$D$5:$D$60,A5,Tasks!$L$5:$L$60,"In progress")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H5" s="65">
         <f>COUNTIFS(Tasks!$D$5:$D$60,A5,Tasks!$L$5:$L$60,"Incident")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I5" t="s">
-        <v>344</v>
+        <v>350</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
@@ -15555,10 +15591,10 @@
         <v>17</v>
       </c>
       <c r="B6" s="65" t="s">
-        <v>345</v>
+        <v>351</v>
       </c>
       <c r="C6" s="65" t="s">
-        <v>346</v>
+        <v>352</v>
       </c>
       <c r="D6" s="65">
         <f>COUNTIFS(Tasks!$D$5:$D$60,A6,Tasks!$B$5:$B$60,"&lt;&gt;P0",Tasks!$A$5:$A$60,"&lt;&gt;WP*")</f>
@@ -15570,18 +15606,18 @@
       </c>
       <c r="F6" s="65">
         <f>COUNTIFS(Tasks!$D$5:$D$60,A6,Tasks!$L$5:$L$60,"Completed",Tasks!$B$5:$B$60,"&lt;&gt;P0")</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G6" s="65">
         <f>COUNTIFS(Tasks!$D$5:$D$60,A6,Tasks!$L$5:$L$60,"In progress")</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H6" s="65">
         <f>COUNTIFS(Tasks!$D$5:$D$60,A6,Tasks!$L$5:$L$60,"Incident")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I6" t="s">
-        <v>347</v>
+        <v>353</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
@@ -15589,10 +15625,10 @@
         <v>13</v>
       </c>
       <c r="B7" s="65" t="s">
-        <v>348</v>
+        <v>354</v>
       </c>
       <c r="C7" s="65" t="s">
-        <v>349</v>
+        <v>355</v>
       </c>
       <c r="D7" s="65">
         <f>COUNTIFS(Tasks!$D$5:$D$60,A7,Tasks!$B$5:$B$60,"&lt;&gt;P0",Tasks!$A$5:$A$60,"&lt;&gt;WP*")</f>
@@ -15604,18 +15640,18 @@
       </c>
       <c r="F7" s="65">
         <f>COUNTIFS(Tasks!$D$5:$D$60,A7,Tasks!$L$5:$L$60,"Completed",Tasks!$B$5:$B$60,"&lt;&gt;P0")</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G7" s="65">
         <f>COUNTIFS(Tasks!$D$5:$D$60,A7,Tasks!$L$5:$L$60,"In progress")</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H7" s="65">
         <f>COUNTIFS(Tasks!$D$5:$D$60,A7,Tasks!$L$5:$L$60,"Incident")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I7" t="s">
-        <v>350</v>
+        <v>356</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
@@ -15623,10 +15659,10 @@
         <v>39</v>
       </c>
       <c r="B8" s="65" t="s">
-        <v>351</v>
+        <v>357</v>
       </c>
       <c r="C8" s="65" t="s">
-        <v>352</v>
+        <v>358</v>
       </c>
       <c r="D8" s="65">
         <f>COUNTIFS(Tasks!$D$5:$D$60,A8,Tasks!$B$5:$B$60,"&lt;&gt;P0",Tasks!$A$5:$A$60,"&lt;&gt;WP*")</f>
@@ -15638,23 +15674,23 @@
       </c>
       <c r="F8" s="65">
         <f>COUNTIFS(Tasks!$D$5:$D$60,A8,Tasks!$L$5:$L$60,"Completed",Tasks!$B$5:$B$60,"&lt;&gt;P0")</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G8" s="65">
         <f>COUNTIFS(Tasks!$D$5:$D$60,A8,Tasks!$L$5:$L$60,"In progress")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H8" s="65">
         <f>COUNTIFS(Tasks!$D$5:$D$60,A8,Tasks!$L$5:$L$60,"Incident")</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I8" t="s">
-        <v>353</v>
+        <v>359</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" s="70" t="s">
-        <v>354</v>
+        <v>360</v>
       </c>
       <c r="D9" s="70">
         <f>SUM(D4:D8)</f>
@@ -15666,7 +15702,7 @@
       </c>
       <c r="F9" s="70">
         <f>SUM(F4:F8)</f>
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="G9" s="70">
         <f>SUM(G4:G8)</f>
@@ -15674,7 +15710,7 @@
       </c>
       <c r="H9" s="70">
         <f>SUM(H4:H8)</f>
-        <v>9</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -15697,33 +15733,33 @@
   <sheetData>
     <row r="1" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="11" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="B1" s="11" t="s">
-        <v>355</v>
+        <v>361</v>
       </c>
       <c r="C1" s="11" t="s">
-        <v>356</v>
+        <v>362</v>
       </c>
       <c r="D1" s="11" t="s">
-        <v>357</v>
+        <v>363</v>
       </c>
       <c r="E1" s="11" t="s">
         <v>9</v>
       </c>
       <c r="F1" s="11" t="s">
-        <v>358</v>
+        <v>364</v>
       </c>
       <c r="G1" s="11" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="65" t="s">
-        <v>359</v>
+        <v>365</v>
       </c>
       <c r="B2" s="65" t="s">
-        <v>360</v>
+        <v>366</v>
       </c>
       <c r="C2" s="71">
         <v>46282</v>
@@ -15735,7 +15771,7 @@
         <v>14</v>
       </c>
       <c r="F2" s="65" t="s">
-        <v>361</v>
+        <v>367</v>
       </c>
       <c r="G2" s="65">
         <f>IF(D2="","",IF(D2&gt;=C2,NETWORKDAYS(C2,D2,Holidays!$A$2:$A$40)-1,-(NETWORKDAYS(D2,C2,Holidays!$A$2:$A$40)-1)))</f>
@@ -15744,10 +15780,10 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="65" t="s">
-        <v>362</v>
+        <v>368</v>
       </c>
       <c r="B3" s="65" t="s">
-        <v>363</v>
+        <v>369</v>
       </c>
       <c r="C3" s="71">
         <v>46304</v>
@@ -15757,7 +15793,7 @@
         <v>51</v>
       </c>
       <c r="F3" s="65" t="s">
-        <v>364</v>
+        <v>370</v>
       </c>
       <c r="G3" s="65" t="str">
         <f>IF(D3="","",IF(D3&gt;=C3,NETWORKDAYS(C3,D3,Holidays!$A$2:$A$40)-1,-(NETWORKDAYS(D3,C3,Holidays!$A$2:$A$40)-1)))</f>
@@ -15766,10 +15802,10 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="65" t="s">
-        <v>365</v>
+        <v>371</v>
       </c>
       <c r="B4" s="65" t="s">
-        <v>366</v>
+        <v>372</v>
       </c>
       <c r="C4" s="71">
         <v>46314</v>
@@ -15779,7 +15815,7 @@
         <v>51</v>
       </c>
       <c r="F4" s="65" t="s">
-        <v>367</v>
+        <v>373</v>
       </c>
       <c r="G4" s="65" t="str">
         <f>IF(D4="","",IF(D4&gt;=C4,NETWORKDAYS(C4,D4,Holidays!$A$2:$A$40)-1,-(NETWORKDAYS(D4,C4,Holidays!$A$2:$A$40)-1)))</f>
@@ -15788,10 +15824,10 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" s="65" t="s">
-        <v>368</v>
+        <v>374</v>
       </c>
       <c r="B5" s="65" t="s">
-        <v>369</v>
+        <v>375</v>
       </c>
       <c r="C5" s="71">
         <v>46316</v>
@@ -15801,7 +15837,7 @@
         <v>51</v>
       </c>
       <c r="F5" s="65" t="s">
-        <v>370</v>
+        <v>376</v>
       </c>
       <c r="G5" s="65" t="str">
         <f>IF(D5="","",IF(D5&gt;=C5,NETWORKDAYS(C5,D5,Holidays!$A$2:$A$40)-1,-(NETWORKDAYS(D5,C5,Holidays!$A$2:$A$40)-1)))</f>
@@ -15810,10 +15846,10 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="65" t="s">
-        <v>371</v>
+        <v>377</v>
       </c>
       <c r="B6" s="65" t="s">
-        <v>372</v>
+        <v>378</v>
       </c>
       <c r="C6" s="71">
         <v>46317</v>
@@ -15823,7 +15859,7 @@
         <v>51</v>
       </c>
       <c r="F6" s="65" t="s">
-        <v>373</v>
+        <v>379</v>
       </c>
       <c r="G6" s="65" t="str">
         <f>IF(D6="","",IF(D6&gt;=C6,NETWORKDAYS(C6,D6,Holidays!$A$2:$A$40)-1,-(NETWORKDAYS(D6,C6,Holidays!$A$2:$A$40)-1)))</f>
@@ -15832,10 +15868,10 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="65" t="s">
-        <v>374</v>
+        <v>380</v>
       </c>
       <c r="B7" s="65" t="s">
-        <v>375</v>
+        <v>381</v>
       </c>
       <c r="C7" s="71">
         <v>46321</v>
@@ -15845,7 +15881,7 @@
         <v>51</v>
       </c>
       <c r="F7" s="65" t="s">
-        <v>376</v>
+        <v>382</v>
       </c>
       <c r="G7" s="65" t="str">
         <f>IF(D7="","",IF(D7&gt;=C7,NETWORKDAYS(C7,D7,Holidays!$A$2:$A$40)-1,-(NETWORKDAYS(D7,C7,Holidays!$A$2:$A$40)-1)))</f>
@@ -15854,10 +15890,10 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" s="65" t="s">
-        <v>377</v>
+        <v>383</v>
       </c>
       <c r="B8" s="65" t="s">
-        <v>378</v>
+        <v>384</v>
       </c>
       <c r="C8" s="71">
         <v>46323</v>
@@ -15867,7 +15903,7 @@
         <v>51</v>
       </c>
       <c r="F8" s="65" t="s">
-        <v>364</v>
+        <v>370</v>
       </c>
       <c r="G8" s="65" t="str">
         <f>IF(D8="","",IF(D8&gt;=C8,NETWORKDAYS(C8,D8,Holidays!$A$2:$A$40)-1,-(NETWORKDAYS(D8,C8,Holidays!$A$2:$A$40)-1)))</f>
@@ -15876,10 +15912,10 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" s="65" t="s">
-        <v>379</v>
+        <v>385</v>
       </c>
       <c r="B9" s="65" t="s">
-        <v>380</v>
+        <v>386</v>
       </c>
       <c r="C9" s="71">
         <v>46331</v>
@@ -15889,7 +15925,7 @@
         <v>51</v>
       </c>
       <c r="F9" s="65" t="s">
-        <v>381</v>
+        <v>387</v>
       </c>
       <c r="G9" s="65" t="str">
         <f>IF(D9="","",IF(D9&gt;=C9,NETWORKDAYS(C9,D9,Holidays!$A$2:$A$40)-1,-(NETWORKDAYS(D9,C9,Holidays!$A$2:$A$40)-1)))</f>
@@ -15925,39 +15961,39 @@
   <sheetData>
     <row r="1" spans="1:11" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="63" t="s">
-        <v>382</v>
+        <v>388</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" s="11" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>383</v>
+        <v>389</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>384</v>
+        <v>390</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>385</v>
+        <v>391</v>
       </c>
       <c r="E3" s="11" t="s">
-        <v>386</v>
+        <v>392</v>
       </c>
       <c r="F3" s="11" t="s">
-        <v>387</v>
+        <v>393</v>
       </c>
       <c r="G3" s="11" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="H3" s="11" t="s">
         <v>9</v>
       </c>
       <c r="I3" s="11" t="s">
-        <v>388</v>
+        <v>394</v>
       </c>
       <c r="J3" s="11" t="s">
-        <v>389</v>
+        <v>395</v>
       </c>
       <c r="K3" s="11" t="s">
         <v>10</v>
@@ -15965,10 +16001,10 @@
     </row>
     <row r="4" spans="1:11" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="74" t="s">
-        <v>390</v>
+        <v>396</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>391</v>
+        <v>397</v>
       </c>
       <c r="C4" s="75">
         <v>2</v>
@@ -15988,24 +16024,24 @@
         <v>17</v>
       </c>
       <c r="H4" s="75" t="s">
-        <v>392</v>
+        <v>398</v>
       </c>
       <c r="I4" s="14" t="s">
-        <v>393</v>
+        <v>399</v>
       </c>
       <c r="J4" s="76">
         <v>46313</v>
       </c>
       <c r="K4" s="19" t="s">
-        <v>394</v>
+        <v>400</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="74" t="s">
-        <v>395</v>
+        <v>401</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>396</v>
+        <v>402</v>
       </c>
       <c r="C5" s="75">
         <v>2</v>
@@ -16025,24 +16061,24 @@
         <v>36</v>
       </c>
       <c r="H5" s="75" t="s">
-        <v>392</v>
+        <v>398</v>
       </c>
       <c r="I5" s="14" t="s">
-        <v>397</v>
+        <v>403</v>
       </c>
       <c r="J5" s="76">
         <v>46313</v>
       </c>
       <c r="K5" s="19" t="s">
-        <v>394</v>
+        <v>400</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="74" t="s">
-        <v>398</v>
+        <v>404</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>399</v>
+        <v>405</v>
       </c>
       <c r="C6" s="75">
         <v>2</v>
@@ -16062,24 +16098,24 @@
         <v>39</v>
       </c>
       <c r="H6" s="75" t="s">
-        <v>392</v>
+        <v>398</v>
       </c>
       <c r="I6" s="14" t="s">
-        <v>400</v>
+        <v>406</v>
       </c>
       <c r="J6" s="76">
         <v>46313</v>
       </c>
       <c r="K6" s="19" t="s">
-        <v>394</v>
+        <v>400</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="74" t="s">
-        <v>401</v>
+        <v>407</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>402</v>
+        <v>408</v>
       </c>
       <c r="C7" s="75">
         <v>3</v>
@@ -16099,24 +16135,24 @@
         <v>13</v>
       </c>
       <c r="H7" s="75" t="s">
-        <v>392</v>
+        <v>398</v>
       </c>
       <c r="I7" s="14" t="s">
-        <v>403</v>
+        <v>409</v>
       </c>
       <c r="J7" s="76">
         <v>46313</v>
       </c>
       <c r="K7" s="19" t="s">
-        <v>394</v>
+        <v>400</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="74" t="s">
-        <v>404</v>
+        <v>410</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>405</v>
+        <v>411</v>
       </c>
       <c r="C8" s="75">
         <v>2</v>
@@ -16136,24 +16172,24 @@
         <v>23</v>
       </c>
       <c r="H8" s="75" t="s">
-        <v>392</v>
+        <v>398</v>
       </c>
       <c r="I8" s="14" t="s">
-        <v>406</v>
+        <v>412</v>
       </c>
       <c r="J8" s="76">
         <v>46313</v>
       </c>
       <c r="K8" s="19" t="s">
-        <v>394</v>
+        <v>400</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="74" t="s">
-        <v>407</v>
+        <v>413</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>408</v>
+        <v>414</v>
       </c>
       <c r="C9" s="75">
         <v>2</v>
@@ -16173,24 +16209,24 @@
         <v>39</v>
       </c>
       <c r="H9" s="75" t="s">
-        <v>392</v>
+        <v>398</v>
       </c>
       <c r="I9" s="14" t="s">
-        <v>409</v>
+        <v>415</v>
       </c>
       <c r="J9" s="76">
         <v>46313</v>
       </c>
       <c r="K9" s="19" t="s">
-        <v>394</v>
+        <v>400</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="74" t="s">
-        <v>410</v>
+        <v>416</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>411</v>
+        <v>417</v>
       </c>
       <c r="C10" s="75">
         <v>1</v>
@@ -16210,24 +16246,24 @@
         <v>17</v>
       </c>
       <c r="H10" s="75" t="s">
-        <v>392</v>
+        <v>398</v>
       </c>
       <c r="I10" s="14" t="s">
-        <v>412</v>
+        <v>418</v>
       </c>
       <c r="J10" s="76">
         <v>46313</v>
       </c>
       <c r="K10" s="19" t="s">
-        <v>394</v>
+        <v>400</v>
       </c>
     </row>
     <row r="11" spans="1:11" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="74" t="s">
-        <v>413</v>
+        <v>419</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>414</v>
+        <v>420</v>
       </c>
       <c r="C11" s="75">
         <v>1</v>
@@ -16247,24 +16283,24 @@
         <v>13</v>
       </c>
       <c r="H11" s="75" t="s">
-        <v>392</v>
+        <v>398</v>
       </c>
       <c r="I11" s="14" t="s">
-        <v>415</v>
+        <v>421</v>
       </c>
       <c r="J11" s="76">
         <v>46313</v>
       </c>
       <c r="K11" s="19" t="s">
-        <v>394</v>
+        <v>400</v>
       </c>
     </row>
     <row r="12" spans="1:11" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="74" t="s">
-        <v>416</v>
+        <v>422</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>417</v>
+        <v>423</v>
       </c>
       <c r="C12" s="75">
         <v>2</v>
@@ -16284,16 +16320,16 @@
         <v>23</v>
       </c>
       <c r="H12" s="75" t="s">
-        <v>392</v>
+        <v>398</v>
       </c>
       <c r="I12" s="14" t="s">
-        <v>418</v>
+        <v>424</v>
       </c>
       <c r="J12" s="76">
         <v>46313</v>
       </c>
       <c r="K12" s="19" t="s">
-        <v>394</v>
+        <v>400</v>
       </c>
     </row>
     <row r="13" spans="1:11" ht="28" customHeight="1" x14ac:dyDescent="0.2">
@@ -16342,10 +16378,10 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="11" t="s">
-        <v>419</v>
+        <v>425</v>
       </c>
       <c r="B1" s="11" t="s">
-        <v>420</v>
+        <v>426</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
@@ -16353,10 +16389,10 @@
         <v>46289</v>
       </c>
       <c r="B2" s="78" t="s">
-        <v>421</v>
+        <v>427</v>
       </c>
       <c r="D2" s="79" t="s">
-        <v>422</v>
+        <v>428</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
@@ -16364,7 +16400,7 @@
         <v>46307</v>
       </c>
       <c r="B3" s="78" t="s">
-        <v>423</v>
+        <v>429</v>
       </c>
     </row>
   </sheetData>

</xml_diff>